<commit_message>
experiments using queueserver or reflectivity
+ configure larch use in config file
+ clarify sync experiment message
+ fix a bug where light xafs_y loads not getting configured
</commit_message>
<xml_diff>
--- a/startup/lookup_table/Modes.xlsx
+++ b/startup/lookup_table/Modes.xlsx
@@ -11830,7 +11830,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:AMJ66"/>
-  <sheetFormatPr defaultColWidth="12.2109375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.2265625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="18.9"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="30.04"/>
@@ -14938,7 +14938,7 @@
         <v>189</v>
       </c>
       <c r="E56" s="60" t="n">
-        <v>122.25</v>
+        <v>120.75</v>
       </c>
       <c r="F56" s="25" t="n">
         <v>9251952</v>
@@ -14950,7 +14950,7 @@
         <v>4600216</v>
       </c>
       <c r="I56" s="60" t="n">
-        <v>56.313</v>
+        <v>54.313</v>
       </c>
       <c r="J56" s="23" t="n">
         <v>6151303</v>
@@ -17154,7 +17154,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="B1:K7"/>
-  <sheetFormatPr defaultColWidth="11.77734375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.78515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="7.34"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="33"/>
@@ -17333,7 +17333,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:I36"/>
-  <sheetFormatPr defaultColWidth="11.77734375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.78515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="17.78"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="11.96"/>
@@ -17685,7 +17685,7 @@
       </c>
       <c r="F23" s="137" t="n">
         <f aca="false">'Modes A-F'!I56</f>
-        <v>56.313</v>
+        <v>54.313</v>
       </c>
       <c r="G23" s="122" t="n">
         <f aca="false">E11-B23*TAN(2*(G19)/1000)+I17</f>
@@ -17904,7 +17904,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:CX484"/>
-  <sheetFormatPr defaultColWidth="11.77734375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.78515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="35.26"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="102" min="2" style="0" width="11.96"/>
@@ -23971,7 +23971,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:G2383"/>
-  <sheetFormatPr defaultColWidth="11.77734375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.78515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="7.05"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="56.14"/>

</xml_diff>

<commit_message>
cleaning up a bunch of recent issues
+ added a function to adjust xafs_table_yu with energy in mode A
+ use tiled better in larch interface
+ publish to kafka with QS
+ reinstall 7 element detector
+ start work on dealing with QS and bsui in kafka consumer: event v. event_page
+ updated lookup table with new values of table motors after a recent
  event in which MC07 lost values
</commit_message>
<xml_diff>
--- a/startup/lookup_table/Modes.xlsx
+++ b/startup/lookup_table/Modes.xlsx
@@ -134,6 +134,19 @@
             <charset val="1"/>
           </rPr>
           <t xml:space="preserve">Position determined at Pt L3 edge</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="E56" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">measured at Cu</t>
         </r>
       </text>
     </comment>
@@ -418,7 +431,9 @@
             <family val="2"/>
             <charset val="1"/>
           </rPr>
-          <t xml:space="preserve">Position determined at Pt L3 edge</t>
+          <t xml:space="preserve">Position determined at Pt L3 edge
+See M3 height
+</t>
         </r>
       </text>
     </comment>
@@ -11830,7 +11845,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:AMJ66"/>
-  <sheetFormatPr defaultColWidth="12.2265625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.25390625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="18.9"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="30.04"/>
@@ -14805,13 +14820,13 @@
         <v>-268324</v>
       </c>
       <c r="K54" s="57" t="n">
-        <v>45.758</v>
+        <v>45.794</v>
       </c>
       <c r="L54" s="28" t="n">
         <v>387964</v>
       </c>
       <c r="M54" s="57" t="n">
-        <v>46.465</v>
+        <v>45.757</v>
       </c>
       <c r="N54" s="28" t="n">
         <v>394647</v>
@@ -14938,7 +14953,7 @@
         <v>189</v>
       </c>
       <c r="E56" s="60" t="n">
-        <v>120.75</v>
+        <v>120.122</v>
       </c>
       <c r="F56" s="25" t="n">
         <v>9251952</v>
@@ -14950,25 +14965,25 @@
         <v>4600216</v>
       </c>
       <c r="I56" s="60" t="n">
-        <v>54.313</v>
+        <v>54.064</v>
       </c>
       <c r="J56" s="23" t="n">
         <v>6151303</v>
       </c>
       <c r="K56" s="60" t="n">
-        <v>130</v>
+        <v>127.868</v>
       </c>
       <c r="L56" s="23" t="n">
         <v>9901395</v>
       </c>
       <c r="M56" s="60" t="n">
-        <v>130.5</v>
+        <v>127.619</v>
       </c>
       <c r="N56" s="23" t="n">
         <v>9901395</v>
       </c>
       <c r="O56" s="60" t="n">
-        <v>101.63</v>
+        <v>99.085</v>
       </c>
       <c r="P56" s="23" t="n">
         <v>8392750</v>
@@ -15000,7 +15015,7 @@
         <v>192</v>
       </c>
       <c r="E57" s="60" t="n">
-        <v>127.288</v>
+        <v>125.022</v>
       </c>
       <c r="F57" s="32" t="n">
         <v>6972005</v>
@@ -15012,25 +15027,25 @@
         <v>1551088</v>
       </c>
       <c r="I57" s="60" t="n">
-        <v>53.237</v>
+        <v>51.187</v>
       </c>
       <c r="J57" s="32" t="n">
         <v>3351899</v>
       </c>
       <c r="K57" s="60" t="n">
-        <v>134.85</v>
+        <v>132.5</v>
       </c>
       <c r="L57" s="32" t="n">
         <v>7552437</v>
       </c>
       <c r="M57" s="60" t="n">
-        <v>136.45</v>
+        <v>132.5</v>
       </c>
       <c r="N57" s="32" t="n">
         <v>7552437</v>
       </c>
       <c r="O57" s="60" t="n">
-        <v>103.067</v>
+        <v>100.567</v>
       </c>
       <c r="P57" s="32" t="n">
         <v>5879304</v>
@@ -15054,7 +15069,7 @@
         <v>195</v>
       </c>
       <c r="E58" s="60" t="n">
-        <v>127.288</v>
+        <v>125.022</v>
       </c>
       <c r="F58" s="28" t="n">
         <v>5572330</v>
@@ -15066,25 +15081,25 @@
         <v>354340</v>
       </c>
       <c r="I58" s="60" t="n">
-        <v>53.237</v>
+        <v>51.187</v>
       </c>
       <c r="J58" s="32" t="n">
         <v>1952224</v>
       </c>
       <c r="K58" s="60" t="n">
-        <v>134.85</v>
+        <v>132.5</v>
       </c>
       <c r="L58" s="32" t="n">
         <v>6355689</v>
       </c>
       <c r="M58" s="60" t="n">
-        <v>136.45</v>
+        <v>132.5</v>
       </c>
       <c r="N58" s="32" t="n">
         <v>6355689</v>
       </c>
       <c r="O58" s="60" t="n">
-        <v>103.067</v>
+        <v>100.567</v>
       </c>
       <c r="P58" s="65" t="n">
         <v>4479629</v>
@@ -17052,7 +17067,7 @@
       </c>
       <c r="F27" s="103" t="n">
         <f aca="false">'Modes A-F'!K54</f>
-        <v>45.758</v>
+        <v>45.794</v>
       </c>
       <c r="G27" s="0"/>
       <c r="H27" s="0"/>
@@ -17071,7 +17086,7 @@
       </c>
       <c r="F28" s="103" t="n">
         <f aca="false">'Modes A-F'!M54</f>
-        <v>46.465</v>
+        <v>45.757</v>
       </c>
       <c r="G28" s="0"/>
       <c r="H28" s="0"/>
@@ -17154,7 +17169,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="B1:K7"/>
-  <sheetFormatPr defaultColWidth="11.78515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.82421875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="7.34"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="33"/>
@@ -17333,7 +17348,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:I36"/>
-  <sheetFormatPr defaultColWidth="11.78515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.82421875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="17.78"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="11.96"/>
@@ -17398,7 +17413,7 @@
       </c>
       <c r="H3" s="122" t="n">
         <f aca="false">G3-F3</f>
-        <v>0.0858810182917011</v>
+        <v>0.0858810182916656</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17414,19 +17429,19 @@
       </c>
       <c r="E4" s="103" t="n">
         <f aca="false">'Modes A-F'!K56</f>
-        <v>130</v>
+        <v>127.868</v>
       </c>
       <c r="F4" s="103" t="n">
         <f aca="false">E4-B4*TAN(2*(F2-E2)/1000)</f>
-        <v>101.088913266688</v>
+        <v>98.9569132666878</v>
       </c>
       <c r="G4" s="121" t="n">
         <f aca="false">'Modes A-F'!O56</f>
-        <v>101.63</v>
+        <v>99.085</v>
       </c>
       <c r="H4" s="122" t="n">
         <f aca="false">G4-F4</f>
-        <v>0.541086733312241</v>
+        <v>0.128086733312244</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17443,25 +17458,25 @@
       </c>
       <c r="E5" s="126" t="n">
         <f aca="false">'Modes A-F'!K57</f>
-        <v>134.85</v>
+        <v>132.5</v>
       </c>
       <c r="F5" s="126" t="n">
         <f aca="false">E5-B5*TAN(2*(F2-E2)/1000)</f>
-        <v>102.47390287165</v>
+        <v>100.12390287165</v>
       </c>
       <c r="G5" s="127" t="n">
         <f aca="false">'Modes A-F'!O57</f>
-        <v>103.067</v>
+        <v>100.567</v>
       </c>
       <c r="H5" s="122" t="n">
         <f aca="false">G5-F5</f>
-        <v>0.593097128349669</v>
+        <v>0.443097128349663</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H6" s="122" t="n">
         <f aca="false">AVERAGE(H3,H4,H5)</f>
-        <v>0.40668829331787</v>
+        <v>0.219021626651191</v>
       </c>
       <c r="I6" s="0" t="s">
         <v>274</v>
@@ -17528,12 +17543,12 @@
       </c>
       <c r="E11" s="122" t="n">
         <f aca="false">'Modes A-F'!E57</f>
-        <v>127.288</v>
+        <v>125.022</v>
       </c>
       <c r="F11" s="122"/>
       <c r="G11" s="131" t="n">
         <f aca="false">E11-B11*TAN(2*(G9-E9)/1000)</f>
-        <v>129.596400030779</v>
+        <v>127.330400030779</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17550,12 +17565,12 @@
       </c>
       <c r="E12" s="132" t="n">
         <f aca="false">'Modes A-F'!E58</f>
-        <v>127.288</v>
+        <v>125.022</v>
       </c>
       <c r="F12" s="132"/>
       <c r="G12" s="133" t="n">
         <f aca="false">E12-B12*TAN(2*(G9-E9)/1000)</f>
-        <v>129.827400033859</v>
+        <v>127.561400033859</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17681,15 +17696,15 @@
       </c>
       <c r="E23" s="122" t="n">
         <f aca="false">E11-B23*TAN(2*(E19)/1000)+I17</f>
-        <v>54.5272674801944</v>
+        <v>52.2612674801944</v>
       </c>
       <c r="F23" s="137" t="n">
         <f aca="false">'Modes A-F'!I56</f>
-        <v>54.313</v>
+        <v>54.064</v>
       </c>
       <c r="G23" s="122" t="n">
         <f aca="false">E11-B23*TAN(2*(G19)/1000)+I17</f>
-        <v>59.8278981480704</v>
+        <v>57.5618981480704</v>
       </c>
       <c r="I23" s="118"/>
     </row>
@@ -17707,15 +17722,15 @@
       </c>
       <c r="E24" s="132" t="n">
         <f aca="false">E12-B24*TAN(2*(E19)/1000)+I17</f>
-        <v>45.8068517843995</v>
+        <v>43.5408517843995</v>
       </c>
       <c r="F24" s="138" t="n">
         <f aca="false">'Modes A-F'!I57</f>
-        <v>53.237</v>
+        <v>51.187</v>
       </c>
       <c r="G24" s="139" t="n">
         <f aca="false">E12-B24*TAN(2*(G19)/1000)+I17</f>
-        <v>51.742766090482</v>
+        <v>49.476766090482</v>
       </c>
       <c r="H24" s="124"/>
       <c r="I24" s="140"/>
@@ -17843,7 +17858,7 @@
       </c>
       <c r="E35" s="122" t="n">
         <f aca="false">E11-B35*TAN(2*(E31)/1000)</f>
-        <v>25.6138777773465</v>
+        <v>23.3478777773465</v>
       </c>
       <c r="F35" s="137" t="n">
         <f aca="false">'Modes A-F'!G56</f>
@@ -17851,7 +17866,7 @@
       </c>
       <c r="G35" s="122" t="n">
         <f aca="false">E11-B35*TAN(2*(G31)/1000)+I29</f>
-        <v>30.9147875381681</v>
+        <v>28.6487875381681</v>
       </c>
       <c r="I35" s="118"/>
     </row>
@@ -17869,7 +17884,7 @@
       </c>
       <c r="E36" s="132" t="n">
         <f aca="false">E12-B36*TAN(2*(E31)/1000)</f>
-        <v>13.428175674289</v>
+        <v>11.162175674289</v>
       </c>
       <c r="F36" s="138" t="n">
         <f aca="false">'Modes A-F'!G57</f>
@@ -17877,7 +17892,7 @@
       </c>
       <c r="G36" s="132" t="n">
         <f aca="false">E12-B36*TAN(2*(G31)/1000)+I29</f>
-        <v>19.3644025227675</v>
+        <v>17.0984025227675</v>
       </c>
       <c r="H36" s="124"/>
       <c r="I36" s="140"/>
@@ -17904,7 +17919,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:CX484"/>
-  <sheetFormatPr defaultColWidth="11.78515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.82421875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="35.26"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="102" min="2" style="0" width="11.96"/>
@@ -23971,7 +23986,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:G2383"/>
-  <sheetFormatPr defaultColWidth="11.78515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.82421875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="7.05"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="56.14"/>

</xml_diff>

<commit_message>
Summer 2026 shutdown activities
+ coupled xafs_ydo and xafs_ydi with eventual intent to add switches
  and encoders.  removed ydo from MODEDATA, renamed ydi to yd.
  Modified XAFSTable to deal with a single downstream motor
+ rewrote pilatus interface to use ROI and Stats plugins correctly
+ same with Eiger sync
+ move XRF plot to kafka
+ moved Mythen mca plot to kafka
+ use toml configuration file in consumer
</commit_message>
<xml_diff>
--- a/startup/lookup_table/Modes.xlsx
+++ b/startup/lookup_table/Modes.xlsx
@@ -66,6 +66,21 @@
             <charset val="1"/>
           </rPr>
           <t xml:space="preserve">Normal operating position is 65 mm – fully out of beam</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="C58" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">August 2026: Couple ydi and ydo after leveling table. Rename ydi → yd. Remove ydo. 
+Remove roll. Will install switches and encoders soon.
+</t>
         </r>
       </text>
     </comment>
@@ -1341,7 +1356,7 @@
     <t xml:space="preserve">XF:06BMA-BI{XAFS-Ax:Tbl_YDI}Mtr</t>
   </si>
   <si>
-    <t xml:space="preserve">xafs_ydi</t>
+    <t xml:space="preserve">xafs_yd</t>
   </si>
   <si>
     <t xml:space="preserve">xafs table ds/ib jack</t>
@@ -10730,7 +10745,7 @@
     <numFmt numFmtId="170" formatCode="yyyy\-mm\-dd"/>
     <numFmt numFmtId="171" formatCode="hh:mm:ss"/>
   </numFmts>
-  <fonts count="19">
+  <fonts count="21">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -10783,6 +10798,20 @@
     <font>
       <vertAlign val="superscript"/>
       <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <color rgb="FFB2B2B2"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FFB2B2B2"/>
       <name val="Arial"/>
       <family val="2"/>
       <charset val="1"/>
@@ -11182,7 +11211,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="146">
+  <cellXfs count="153">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -11435,6 +11464,34 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="10" fillId="7" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="7" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="166" fontId="0" fillId="7" borderId="6" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -11511,87 +11568,87 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="8" borderId="25" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="8" borderId="25" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="26" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="26" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="27" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="27" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="27" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="27" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="28" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="28" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="29" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="29" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="30" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="30" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="8" borderId="25" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="8" borderId="25" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="26" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="26" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="26" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="26" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="27" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="27" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="27" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="27" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -11599,27 +11656,27 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -11635,7 +11692,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="16" fillId="0" borderId="32" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="18" fillId="0" borderId="32" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -11695,7 +11752,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="16" fillId="0" borderId="31" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="18" fillId="0" borderId="31" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -11723,7 +11780,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -11747,7 +11804,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="18" fillId="0" borderId="31" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="20" fillId="0" borderId="31" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -11825,7 +11882,7 @@
       <rgbColor rgb="FFFF9900"/>
       <rgbColor rgb="FFFF6600"/>
       <rgbColor rgb="FF666699"/>
-      <rgbColor rgb="FF969696"/>
+      <rgbColor rgb="FFB2B2B2"/>
       <rgbColor rgb="FF003366"/>
       <rgbColor rgb="FF339966"/>
       <rgbColor rgb="FF003300"/>
@@ -11845,7 +11902,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:AMJ66"/>
-  <sheetFormatPr defaultColWidth="12.25390625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.2734375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="18.9"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="30.04"/>
@@ -15003,57 +15060,57 @@
       <c r="Y56" s="0"/>
       <c r="Z56" s="0"/>
     </row>
-    <row r="57" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="57" s="64" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="18"/>
-      <c r="B57" s="44" t="s">
+      <c r="B57" s="63" t="s">
         <v>190</v>
       </c>
-      <c r="C57" s="0" t="s">
+      <c r="C57" s="64" t="s">
         <v>191</v>
       </c>
-      <c r="D57" s="0" t="s">
+      <c r="D57" s="64" t="s">
         <v>192</v>
       </c>
-      <c r="E57" s="60" t="n">
+      <c r="E57" s="65" t="n">
         <v>125.022</v>
       </c>
-      <c r="F57" s="32" t="n">
+      <c r="F57" s="66" t="n">
         <v>6972005</v>
       </c>
-      <c r="G57" s="63" t="n">
+      <c r="G57" s="67" t="n">
         <v>12.81</v>
       </c>
-      <c r="H57" s="64" t="n">
+      <c r="H57" s="68" t="n">
         <v>1551088</v>
       </c>
-      <c r="I57" s="60" t="n">
+      <c r="I57" s="65" t="n">
         <v>51.187</v>
       </c>
-      <c r="J57" s="32" t="n">
+      <c r="J57" s="66" t="n">
         <v>3351899</v>
       </c>
-      <c r="K57" s="60" t="n">
+      <c r="K57" s="65" t="n">
         <v>132.5</v>
       </c>
-      <c r="L57" s="32" t="n">
+      <c r="L57" s="66" t="n">
         <v>7552437</v>
       </c>
-      <c r="M57" s="60" t="n">
+      <c r="M57" s="65" t="n">
         <v>132.5</v>
       </c>
-      <c r="N57" s="32" t="n">
+      <c r="N57" s="66" t="n">
         <v>7552437</v>
       </c>
-      <c r="O57" s="60" t="n">
+      <c r="O57" s="65" t="n">
         <v>100.567</v>
       </c>
-      <c r="P57" s="32" t="n">
+      <c r="P57" s="66" t="n">
         <v>5879304</v>
       </c>
-      <c r="T57" s="55" t="n">
+      <c r="T57" s="69" t="n">
         <v>143.4</v>
       </c>
-      <c r="U57" s="32" t="n">
+      <c r="U57" s="66" t="n">
         <v>8085853</v>
       </c>
     </row>
@@ -15074,10 +15131,10 @@
       <c r="F58" s="28" t="n">
         <v>5572330</v>
       </c>
-      <c r="G58" s="63" t="n">
+      <c r="G58" s="70" t="n">
         <v>12.81</v>
       </c>
-      <c r="H58" s="64" t="n">
+      <c r="H58" s="71" t="n">
         <v>354340</v>
       </c>
       <c r="I58" s="60" t="n">
@@ -15101,7 +15158,7 @@
       <c r="O58" s="60" t="n">
         <v>100.567</v>
       </c>
-      <c r="P58" s="65" t="n">
+      <c r="P58" s="72" t="n">
         <v>4479629</v>
       </c>
       <c r="T58" s="55" t="n">
@@ -15127,43 +15184,43 @@
       <c r="D59" s="26" t="s">
         <v>198</v>
       </c>
-      <c r="E59" s="66" t="n">
+      <c r="E59" s="73" t="n">
         <v>-9.0621</v>
       </c>
       <c r="F59" s="28" t="n">
         <v>-242758</v>
       </c>
-      <c r="G59" s="63" t="n">
+      <c r="G59" s="70" t="n">
         <v>-9.0621</v>
       </c>
-      <c r="H59" s="67" t="n">
+      <c r="H59" s="74" t="n">
         <v>-242758</v>
       </c>
-      <c r="I59" s="66" t="n">
+      <c r="I59" s="73" t="n">
         <v>-9.0621</v>
       </c>
       <c r="J59" s="28" t="n">
         <v>-242758</v>
       </c>
-      <c r="K59" s="66" t="n">
+      <c r="K59" s="73" t="n">
         <v>-9.0621</v>
       </c>
       <c r="L59" s="28" t="n">
         <v>-242758</v>
       </c>
-      <c r="M59" s="66" t="n">
+      <c r="M59" s="73" t="n">
         <v>-9.0621</v>
       </c>
       <c r="N59" s="28" t="n">
         <v>-242758</v>
       </c>
-      <c r="O59" s="66" t="n">
+      <c r="O59" s="73" t="n">
         <v>-9.0621</v>
       </c>
       <c r="P59" s="28" t="n">
         <v>-242758</v>
       </c>
-      <c r="T59" s="66" t="n">
+      <c r="T59" s="73" t="n">
         <v>-0.6</v>
       </c>
       <c r="U59" s="28" t="n">
@@ -15181,46 +15238,46 @@
       <c r="D60" s="35" t="s">
         <v>201</v>
       </c>
-      <c r="E60" s="68" t="n">
+      <c r="E60" s="75" t="n">
         <v>15.3898</v>
       </c>
       <c r="F60" s="47" t="n">
         <v>160203</v>
       </c>
-      <c r="G60" s="69" t="n">
+      <c r="G60" s="76" t="n">
         <v>15.3898</v>
       </c>
-      <c r="H60" s="70" t="n">
+      <c r="H60" s="77" t="n">
         <v>160203</v>
       </c>
-      <c r="I60" s="68" t="n">
+      <c r="I60" s="75" t="n">
         <v>15.3898</v>
       </c>
       <c r="J60" s="47" t="n">
         <v>160203</v>
       </c>
-      <c r="K60" s="68" t="n">
+      <c r="K60" s="75" t="n">
         <v>15.3898</v>
       </c>
       <c r="L60" s="47" t="n">
         <v>160203</v>
       </c>
-      <c r="M60" s="68" t="n">
+      <c r="M60" s="75" t="n">
         <v>15.3898</v>
       </c>
       <c r="N60" s="47" t="n">
         <v>160203</v>
       </c>
-      <c r="O60" s="68" t="n">
+      <c r="O60" s="75" t="n">
         <v>15.3898</v>
       </c>
       <c r="P60" s="47" t="n">
         <v>160203</v>
       </c>
-      <c r="Q60" s="71"/>
-      <c r="R60" s="71"/>
-      <c r="S60" s="71"/>
-      <c r="T60" s="68" t="n">
+      <c r="Q60" s="78"/>
+      <c r="R60" s="78"/>
+      <c r="S60" s="78"/>
+      <c r="T60" s="75" t="n">
         <v>33.3721</v>
       </c>
       <c r="U60" s="47" t="n">
@@ -15233,52 +15290,52 @@
       <c r="Z60" s="0"/>
     </row>
     <row r="61" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A61" s="72" t="s">
+      <c r="A61" s="79" t="s">
         <v>202</v>
       </c>
-      <c r="B61" s="73" t="s">
+      <c r="B61" s="80" t="s">
         <v>203</v>
       </c>
-      <c r="C61" s="74" t="s">
+      <c r="C61" s="81" t="s">
         <v>204</v>
       </c>
-      <c r="D61" s="74" t="s">
+      <c r="D61" s="81" t="s">
         <v>205</v>
       </c>
-      <c r="E61" s="75" t="n">
-        <v>0</v>
-      </c>
-      <c r="F61" s="76" t="n">
-        <v>0</v>
-      </c>
-      <c r="G61" s="75" t="n">
-        <v>0</v>
-      </c>
-      <c r="H61" s="76" t="n">
-        <v>0</v>
-      </c>
-      <c r="I61" s="75" t="n">
-        <v>0</v>
-      </c>
-      <c r="J61" s="76" t="n">
-        <v>0</v>
-      </c>
-      <c r="K61" s="75" t="n">
-        <v>0</v>
-      </c>
-      <c r="L61" s="76" t="n">
-        <v>0</v>
-      </c>
-      <c r="M61" s="75" t="n">
-        <v>0</v>
-      </c>
-      <c r="N61" s="76" t="n">
-        <v>0</v>
-      </c>
-      <c r="O61" s="75" t="n">
-        <v>0</v>
-      </c>
-      <c r="P61" s="76" t="n">
+      <c r="E61" s="82" t="n">
+        <v>0</v>
+      </c>
+      <c r="F61" s="83" t="n">
+        <v>0</v>
+      </c>
+      <c r="G61" s="82" t="n">
+        <v>0</v>
+      </c>
+      <c r="H61" s="83" t="n">
+        <v>0</v>
+      </c>
+      <c r="I61" s="82" t="n">
+        <v>0</v>
+      </c>
+      <c r="J61" s="83" t="n">
+        <v>0</v>
+      </c>
+      <c r="K61" s="82" t="n">
+        <v>0</v>
+      </c>
+      <c r="L61" s="83" t="n">
+        <v>0</v>
+      </c>
+      <c r="M61" s="82" t="n">
+        <v>0</v>
+      </c>
+      <c r="N61" s="83" t="n">
+        <v>0</v>
+      </c>
+      <c r="O61" s="82" t="n">
+        <v>0</v>
+      </c>
+      <c r="P61" s="83" t="n">
         <v>0</v>
       </c>
       <c r="T61" s="30" t="n">
@@ -15289,8 +15346,8 @@
       </c>
     </row>
     <row r="62" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A62" s="72"/>
-      <c r="B62" s="77" t="s">
+      <c r="A62" s="79"/>
+      <c r="B62" s="84" t="s">
         <v>206</v>
       </c>
       <c r="C62" s="0" t="s">
@@ -15343,8 +15400,8 @@
       </c>
     </row>
     <row r="63" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A63" s="72"/>
-      <c r="B63" s="77" t="s">
+      <c r="A63" s="79"/>
+      <c r="B63" s="84" t="s">
         <v>209</v>
       </c>
       <c r="C63" s="0" t="s">
@@ -15397,8 +15454,8 @@
       </c>
     </row>
     <row r="64" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A64" s="72"/>
-      <c r="B64" s="77" t="s">
+      <c r="A64" s="79"/>
+      <c r="B64" s="84" t="s">
         <v>212</v>
       </c>
       <c r="C64" s="0" t="s">
@@ -15451,8 +15508,8 @@
       </c>
     </row>
     <row r="65" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A65" s="72"/>
-      <c r="B65" s="77" t="s">
+      <c r="A65" s="79"/>
+      <c r="B65" s="84" t="s">
         <v>215</v>
       </c>
       <c r="C65" s="0" t="s">
@@ -15505,53 +15562,53 @@
       </c>
     </row>
     <row r="66" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A66" s="72"/>
-      <c r="B66" s="78" t="s">
+      <c r="A66" s="79"/>
+      <c r="B66" s="85" t="s">
         <v>218</v>
       </c>
-      <c r="C66" s="79" t="s">
+      <c r="C66" s="86" t="s">
         <v>219</v>
       </c>
-      <c r="D66" s="79" t="s">
+      <c r="D66" s="86" t="s">
         <v>220</v>
       </c>
-      <c r="E66" s="80" t="n">
-        <v>0</v>
-      </c>
-      <c r="F66" s="81" t="n">
-        <v>0</v>
-      </c>
-      <c r="G66" s="80" t="n">
-        <v>0</v>
-      </c>
-      <c r="H66" s="81" t="n">
-        <v>0</v>
-      </c>
-      <c r="I66" s="80" t="n">
-        <v>0</v>
-      </c>
-      <c r="J66" s="81" t="n">
-        <v>0</v>
-      </c>
-      <c r="K66" s="80" t="n">
-        <v>0</v>
-      </c>
-      <c r="L66" s="81" t="n">
-        <v>0</v>
-      </c>
-      <c r="M66" s="80" t="n">
-        <v>0</v>
-      </c>
-      <c r="N66" s="81" t="n">
-        <v>0</v>
-      </c>
-      <c r="O66" s="80" t="n">
-        <v>0</v>
-      </c>
-      <c r="P66" s="81" t="n">
-        <v>0</v>
-      </c>
-      <c r="T66" s="68" t="n">
+      <c r="E66" s="87" t="n">
+        <v>0</v>
+      </c>
+      <c r="F66" s="88" t="n">
+        <v>0</v>
+      </c>
+      <c r="G66" s="87" t="n">
+        <v>0</v>
+      </c>
+      <c r="H66" s="88" t="n">
+        <v>0</v>
+      </c>
+      <c r="I66" s="87" t="n">
+        <v>0</v>
+      </c>
+      <c r="J66" s="88" t="n">
+        <v>0</v>
+      </c>
+      <c r="K66" s="87" t="n">
+        <v>0</v>
+      </c>
+      <c r="L66" s="88" t="n">
+        <v>0</v>
+      </c>
+      <c r="M66" s="87" t="n">
+        <v>0</v>
+      </c>
+      <c r="N66" s="88" t="n">
+        <v>0</v>
+      </c>
+      <c r="O66" s="87" t="n">
+        <v>0</v>
+      </c>
+      <c r="P66" s="88" t="n">
+        <v>0</v>
+      </c>
+      <c r="T66" s="75" t="n">
         <v>0</v>
       </c>
       <c r="U66" s="47" t="n">
@@ -15606,34 +15663,34 @@
   <dimension ref="A1:AMJ31"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="82" width="3.11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="2" style="82" width="13.26"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1024" min="10" style="82" width="11.52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="89" width="3.11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="2" style="89" width="13.26"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1024" min="10" style="89" width="11.52"/>
   </cols>
   <sheetData>
-    <row r="1" s="83" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="82"/>
+    <row r="1" s="90" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="89"/>
       <c r="B1" s="0"/>
       <c r="C1" s="0"/>
       <c r="D1" s="0"/>
       <c r="E1" s="0"/>
-      <c r="F1" s="82"/>
-      <c r="G1" s="82"/>
-      <c r="H1" s="82"/>
-      <c r="I1" s="82"/>
-      <c r="J1" s="82"/>
-      <c r="K1" s="82"/>
-      <c r="L1" s="82"/>
-      <c r="AMJ1" s="82"/>
+      <c r="F1" s="89"/>
+      <c r="G1" s="89"/>
+      <c r="H1" s="89"/>
+      <c r="I1" s="89"/>
+      <c r="J1" s="89"/>
+      <c r="K1" s="89"/>
+      <c r="L1" s="89"/>
+      <c r="AMJ1" s="89"/>
     </row>
     <row r="2" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0"/>
-      <c r="B2" s="84" t="s">
+      <c r="B2" s="91" t="s">
         <v>221</v>
       </c>
-      <c r="C2" s="84"/>
-      <c r="D2" s="84"/>
-      <c r="E2" s="84"/>
+      <c r="C2" s="91"/>
+      <c r="D2" s="91"/>
+      <c r="E2" s="91"/>
       <c r="F2" s="0"/>
       <c r="G2" s="0"/>
       <c r="H2" s="0"/>
@@ -16654,168 +16711,168 @@
       <c r="AMI2" s="0"/>
       <c r="AMJ2" s="0"/>
     </row>
-    <row r="3" s="89" customFormat="true" ht="25.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="85"/>
-      <c r="B3" s="86"/>
-      <c r="C3" s="87" t="s">
+    <row r="3" s="96" customFormat="true" ht="25.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="92"/>
+      <c r="B3" s="93"/>
+      <c r="C3" s="94" t="s">
         <v>222</v>
       </c>
-      <c r="D3" s="87" t="s">
+      <c r="D3" s="94" t="s">
         <v>223</v>
       </c>
-      <c r="E3" s="88" t="s">
+      <c r="E3" s="95" t="s">
         <v>224</v>
       </c>
-      <c r="F3" s="85"/>
-      <c r="G3" s="85"/>
-      <c r="H3" s="85"/>
-      <c r="I3" s="85"/>
-      <c r="J3" s="85"/>
-      <c r="K3" s="85"/>
-      <c r="L3" s="85"/>
-      <c r="AMJ3" s="85"/>
-    </row>
-    <row r="4" s="83" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="82"/>
-      <c r="B4" s="86" t="s">
+      <c r="F3" s="92"/>
+      <c r="G3" s="92"/>
+      <c r="H3" s="92"/>
+      <c r="I3" s="92"/>
+      <c r="J3" s="92"/>
+      <c r="K3" s="92"/>
+      <c r="L3" s="92"/>
+      <c r="AMJ3" s="92"/>
+    </row>
+    <row r="4" s="90" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="89"/>
+      <c r="B4" s="93" t="s">
         <v>225</v>
       </c>
-      <c r="C4" s="82"/>
-      <c r="D4" s="82" t="n">
+      <c r="C4" s="89"/>
+      <c r="D4" s="89" t="n">
         <v>55</v>
       </c>
-      <c r="E4" s="90" t="n">
+      <c r="E4" s="97" t="n">
         <v>55</v>
       </c>
-      <c r="F4" s="82"/>
-      <c r="G4" s="82"/>
-      <c r="H4" s="82"/>
-      <c r="I4" s="82"/>
-      <c r="J4" s="82"/>
-      <c r="K4" s="82"/>
-      <c r="L4" s="82"/>
-      <c r="AMJ4" s="82"/>
-    </row>
-    <row r="5" s="83" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="82"/>
-      <c r="B5" s="86" t="s">
+      <c r="F4" s="89"/>
+      <c r="G4" s="89"/>
+      <c r="H4" s="89"/>
+      <c r="I4" s="89"/>
+      <c r="J4" s="89"/>
+      <c r="K4" s="89"/>
+      <c r="L4" s="89"/>
+      <c r="AMJ4" s="89"/>
+    </row>
+    <row r="5" s="90" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="89"/>
+      <c r="B5" s="93" t="s">
         <v>226</v>
       </c>
-      <c r="C5" s="82" t="s">
+      <c r="C5" s="89" t="s">
         <v>227</v>
       </c>
-      <c r="D5" s="82" t="n">
+      <c r="D5" s="89" t="n">
         <v>-46.5</v>
       </c>
-      <c r="E5" s="90"/>
-      <c r="F5" s="82"/>
-      <c r="G5" s="82"/>
-      <c r="H5" s="82"/>
-      <c r="I5" s="82"/>
-      <c r="J5" s="82"/>
-      <c r="K5" s="82"/>
-      <c r="L5" s="82"/>
-      <c r="AMJ5" s="82"/>
-    </row>
-    <row r="6" s="83" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="82"/>
-      <c r="B6" s="86" t="s">
+      <c r="E5" s="97"/>
+      <c r="F5" s="89"/>
+      <c r="G5" s="89"/>
+      <c r="H5" s="89"/>
+      <c r="I5" s="89"/>
+      <c r="J5" s="89"/>
+      <c r="K5" s="89"/>
+      <c r="L5" s="89"/>
+      <c r="AMJ5" s="89"/>
+    </row>
+    <row r="6" s="90" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="89"/>
+      <c r="B6" s="93" t="s">
         <v>228</v>
       </c>
-      <c r="C6" s="82" t="s">
+      <c r="C6" s="89" t="s">
         <v>229</v>
       </c>
-      <c r="D6" s="82" t="n">
+      <c r="D6" s="89" t="n">
         <v>-20.5</v>
       </c>
-      <c r="E6" s="90"/>
-      <c r="F6" s="82"/>
-      <c r="G6" s="82"/>
-      <c r="H6" s="82"/>
-      <c r="I6" s="82"/>
-      <c r="J6" s="82"/>
-      <c r="K6" s="82"/>
-      <c r="L6" s="82"/>
-      <c r="AMJ6" s="82"/>
-    </row>
-    <row r="7" s="83" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="82"/>
-      <c r="B7" s="86" t="s">
+      <c r="E6" s="97"/>
+      <c r="F6" s="89"/>
+      <c r="G6" s="89"/>
+      <c r="H6" s="89"/>
+      <c r="I6" s="89"/>
+      <c r="J6" s="89"/>
+      <c r="K6" s="89"/>
+      <c r="L6" s="89"/>
+      <c r="AMJ6" s="89"/>
+    </row>
+    <row r="7" s="90" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="89"/>
+      <c r="B7" s="93" t="s">
         <v>230</v>
       </c>
-      <c r="C7" s="82" t="s">
+      <c r="C7" s="89" t="s">
         <v>231</v>
       </c>
-      <c r="D7" s="82" t="n">
+      <c r="D7" s="89" t="n">
         <v>5.5</v>
       </c>
-      <c r="E7" s="90"/>
-      <c r="F7" s="82"/>
-      <c r="G7" s="82"/>
-      <c r="H7" s="82"/>
-      <c r="I7" s="82"/>
-      <c r="J7" s="82"/>
-      <c r="K7" s="82"/>
-      <c r="L7" s="82"/>
-      <c r="AMJ7" s="82"/>
-    </row>
-    <row r="8" s="83" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="82"/>
-      <c r="B8" s="86" t="s">
+      <c r="E7" s="97"/>
+      <c r="F7" s="89"/>
+      <c r="G7" s="89"/>
+      <c r="H7" s="89"/>
+      <c r="I7" s="89"/>
+      <c r="J7" s="89"/>
+      <c r="K7" s="89"/>
+      <c r="L7" s="89"/>
+      <c r="AMJ7" s="89"/>
+    </row>
+    <row r="8" s="90" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="89"/>
+      <c r="B8" s="93" t="s">
         <v>232</v>
       </c>
-      <c r="C8" s="82" t="s">
+      <c r="C8" s="89" t="s">
         <v>233</v>
       </c>
-      <c r="D8" s="82" t="n">
+      <c r="D8" s="89" t="n">
         <v>31</v>
       </c>
-      <c r="E8" s="90"/>
-      <c r="F8" s="82"/>
-      <c r="G8" s="82"/>
-      <c r="H8" s="82"/>
-      <c r="I8" s="82"/>
-      <c r="J8" s="82"/>
-      <c r="K8" s="82"/>
-      <c r="L8" s="82"/>
-      <c r="AMJ8" s="82"/>
-    </row>
-    <row r="9" s="83" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="82"/>
-      <c r="B9" s="86" t="s">
+      <c r="E8" s="97"/>
+      <c r="F8" s="89"/>
+      <c r="G8" s="89"/>
+      <c r="H8" s="89"/>
+      <c r="I8" s="89"/>
+      <c r="J8" s="89"/>
+      <c r="K8" s="89"/>
+      <c r="L8" s="89"/>
+      <c r="AMJ8" s="89"/>
+    </row>
+    <row r="9" s="90" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="89"/>
+      <c r="B9" s="93" t="s">
         <v>234</v>
       </c>
-      <c r="C9" s="82"/>
-      <c r="D9" s="82" t="n">
+      <c r="C9" s="89"/>
+      <c r="D9" s="89" t="n">
         <v>-52.6</v>
       </c>
-      <c r="E9" s="90"/>
-      <c r="F9" s="82"/>
-      <c r="G9" s="82"/>
-      <c r="H9" s="82"/>
-      <c r="I9" s="82"/>
-      <c r="J9" s="82"/>
-      <c r="K9" s="82"/>
-      <c r="L9" s="82"/>
-      <c r="AMJ9" s="82"/>
+      <c r="E9" s="97"/>
+      <c r="F9" s="89"/>
+      <c r="G9" s="89"/>
+      <c r="H9" s="89"/>
+      <c r="I9" s="89"/>
+      <c r="J9" s="89"/>
+      <c r="K9" s="89"/>
+      <c r="L9" s="89"/>
+      <c r="AMJ9" s="89"/>
     </row>
     <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B10" s="91" t="s">
+      <c r="B10" s="98" t="s">
         <v>235</v>
       </c>
-      <c r="C10" s="92"/>
-      <c r="D10" s="92" t="n">
+      <c r="C10" s="99"/>
+      <c r="D10" s="99" t="n">
         <v>-52</v>
       </c>
-      <c r="E10" s="93"/>
+      <c r="E10" s="100"/>
       <c r="F10" s="0"/>
       <c r="G10" s="0"/>
       <c r="H10" s="0"/>
       <c r="I10" s="0"/>
     </row>
     <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B11" s="94"/>
-      <c r="C11" s="95"/>
+      <c r="B11" s="101"/>
+      <c r="C11" s="102"/>
       <c r="D11" s="0"/>
       <c r="E11" s="0"/>
       <c r="F11" s="0"/>
@@ -16824,8 +16881,8 @@
       <c r="I11" s="0"/>
     </row>
     <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B12" s="94"/>
-      <c r="C12" s="95"/>
+      <c r="B12" s="101"/>
+      <c r="C12" s="102"/>
       <c r="D12" s="0"/>
       <c r="E12" s="0"/>
       <c r="F12" s="0"/>
@@ -16834,82 +16891,82 @@
       <c r="I12" s="0"/>
     </row>
     <row r="13" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B13" s="96" t="s">
+      <c r="B13" s="103" t="s">
         <v>236</v>
       </c>
-      <c r="C13" s="96"/>
-      <c r="D13" s="96"/>
-      <c r="E13" s="96"/>
+      <c r="C13" s="103"/>
+      <c r="D13" s="103"/>
+      <c r="E13" s="103"/>
       <c r="F13" s="0"/>
       <c r="G13" s="0"/>
       <c r="H13" s="0"/>
       <c r="I13" s="0"/>
     </row>
     <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B14" s="97" t="s">
+      <c r="B14" s="104" t="s">
         <v>237</v>
       </c>
-      <c r="C14" s="98" t="s">
+      <c r="C14" s="105" t="s">
         <v>238</v>
       </c>
       <c r="D14" s="0"/>
-      <c r="E14" s="90"/>
+      <c r="E14" s="97"/>
       <c r="F14" s="0"/>
       <c r="G14" s="0"/>
       <c r="H14" s="0"/>
       <c r="I14" s="0"/>
     </row>
     <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B15" s="86" t="s">
+      <c r="B15" s="93" t="s">
         <v>225</v>
       </c>
-      <c r="C15" s="82" t="n">
+      <c r="C15" s="89" t="n">
         <v>67</v>
       </c>
       <c r="D15" s="0"/>
-      <c r="E15" s="90"/>
+      <c r="E15" s="97"/>
       <c r="F15" s="0"/>
       <c r="G15" s="0"/>
       <c r="H15" s="0"/>
       <c r="I15" s="0"/>
     </row>
     <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B16" s="86" t="s">
+      <c r="B16" s="93" t="s">
         <v>239</v>
       </c>
-      <c r="C16" s="99" t="n">
+      <c r="C16" s="106" t="n">
         <v>-1.5</v>
       </c>
       <c r="D16" s="0"/>
-      <c r="E16" s="90"/>
+      <c r="E16" s="97"/>
       <c r="F16" s="0"/>
       <c r="G16" s="0"/>
       <c r="H16" s="0"/>
       <c r="I16" s="0"/>
     </row>
     <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B17" s="86" t="s">
+      <c r="B17" s="93" t="s">
         <v>240</v>
       </c>
-      <c r="C17" s="82" t="n">
+      <c r="C17" s="89" t="n">
         <v>33</v>
       </c>
       <c r="D17" s="0"/>
-      <c r="E17" s="90"/>
+      <c r="E17" s="97"/>
       <c r="F17" s="0"/>
       <c r="G17" s="0"/>
       <c r="H17" s="0"/>
       <c r="I17" s="0"/>
     </row>
     <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B18" s="91" t="s">
+      <c r="B18" s="98" t="s">
         <v>241</v>
       </c>
-      <c r="C18" s="92" t="n">
+      <c r="C18" s="99" t="n">
         <v>53</v>
       </c>
-      <c r="D18" s="92"/>
-      <c r="E18" s="93"/>
+      <c r="D18" s="99"/>
+      <c r="E18" s="100"/>
       <c r="F18" s="0"/>
       <c r="G18" s="0"/>
       <c r="H18" s="0"/>
@@ -16936,213 +16993,213 @@
       <c r="I20" s="0"/>
     </row>
     <row r="21" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B21" s="96" t="s">
+      <c r="B21" s="103" t="s">
         <v>176</v>
       </c>
-      <c r="C21" s="96"/>
-      <c r="D21" s="96"/>
-      <c r="E21" s="96"/>
-      <c r="F21" s="96"/>
-      <c r="G21" s="96"/>
-      <c r="H21" s="96"/>
-      <c r="I21" s="96"/>
+      <c r="C21" s="103"/>
+      <c r="D21" s="103"/>
+      <c r="E21" s="103"/>
+      <c r="F21" s="103"/>
+      <c r="G21" s="103"/>
+      <c r="H21" s="103"/>
+      <c r="I21" s="103"/>
     </row>
     <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B22" s="100" t="s">
+      <c r="B22" s="107" t="s">
         <v>242</v>
       </c>
-      <c r="C22" s="100"/>
-      <c r="D22" s="83"/>
-      <c r="E22" s="94" t="s">
+      <c r="C22" s="107"/>
+      <c r="D22" s="90"/>
+      <c r="E22" s="101" t="s">
         <v>243</v>
       </c>
-      <c r="F22" s="94"/>
-      <c r="G22" s="83"/>
-      <c r="H22" s="101" t="s">
+      <c r="F22" s="101"/>
+      <c r="G22" s="90"/>
+      <c r="H22" s="108" t="s">
         <v>244</v>
       </c>
-      <c r="I22" s="101"/>
+      <c r="I22" s="108"/>
     </row>
     <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B23" s="97" t="s">
+      <c r="B23" s="104" t="s">
         <v>245</v>
       </c>
-      <c r="C23" s="98" t="s">
+      <c r="C23" s="105" t="s">
         <v>238</v>
       </c>
       <c r="D23" s="0"/>
-      <c r="E23" s="83" t="s">
+      <c r="E23" s="90" t="s">
         <v>245</v>
       </c>
-      <c r="F23" s="98" t="s">
+      <c r="F23" s="105" t="s">
         <v>238</v>
       </c>
       <c r="G23" s="0"/>
-      <c r="H23" s="83" t="s">
+      <c r="H23" s="90" t="s">
         <v>246</v>
       </c>
-      <c r="I23" s="102" t="s">
+      <c r="I23" s="109" t="s">
         <v>238</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B24" s="86" t="s">
+      <c r="B24" s="93" t="s">
         <v>247</v>
       </c>
       <c r="C24" s="0" t="n">
         <v>33</v>
       </c>
       <c r="D24" s="0"/>
-      <c r="E24" s="82" t="s">
+      <c r="E24" s="89" t="s">
         <v>247</v>
       </c>
-      <c r="F24" s="103" t="n">
+      <c r="F24" s="110" t="n">
         <f aca="false">'Modes A-F'!E54</f>
         <v>37.717</v>
       </c>
       <c r="G24" s="0"/>
-      <c r="H24" s="82" t="s">
+      <c r="H24" s="89" t="s">
         <v>248</v>
       </c>
-      <c r="I24" s="90" t="n">
+      <c r="I24" s="97" t="n">
         <v>40</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B25" s="86" t="s">
+      <c r="B25" s="93" t="s">
         <v>249</v>
       </c>
       <c r="C25" s="0" t="n">
         <v>-66.743</v>
       </c>
       <c r="D25" s="0"/>
-      <c r="E25" s="82" t="s">
+      <c r="E25" s="89" t="s">
         <v>249</v>
       </c>
-      <c r="F25" s="103" t="n">
+      <c r="F25" s="110" t="n">
         <f aca="false">'Modes A-F'!G54</f>
         <v>-55.188</v>
       </c>
       <c r="G25" s="0"/>
-      <c r="H25" s="82" t="s">
+      <c r="H25" s="89" t="s">
         <v>250</v>
       </c>
-      <c r="I25" s="90" t="n">
+      <c r="I25" s="97" t="n">
         <v>-17.5</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B26" s="86" t="s">
+      <c r="B26" s="93" t="s">
         <v>251</v>
       </c>
       <c r="C26" s="0" t="n">
         <v>-48.1824</v>
       </c>
       <c r="D26" s="0"/>
-      <c r="E26" s="82" t="s">
+      <c r="E26" s="89" t="s">
         <v>251</v>
       </c>
-      <c r="F26" s="103" t="n">
+      <c r="F26" s="110" t="n">
         <f aca="false">'Modes A-F'!I54</f>
         <v>-23.201</v>
       </c>
       <c r="G26" s="0"/>
-      <c r="H26" s="82" t="s">
+      <c r="H26" s="89" t="s">
         <v>252</v>
       </c>
-      <c r="I26" s="90" t="n">
+      <c r="I26" s="97" t="n">
         <v>6.5</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B27" s="86" t="s">
+      <c r="B27" s="93" t="s">
         <v>253</v>
       </c>
-      <c r="C27" s="82" t="n">
+      <c r="C27" s="89" t="n">
         <v>27.1</v>
       </c>
       <c r="D27" s="0"/>
-      <c r="E27" s="82" t="s">
+      <c r="E27" s="89" t="s">
         <v>253</v>
       </c>
-      <c r="F27" s="103" t="n">
+      <c r="F27" s="110" t="n">
         <f aca="false">'Modes A-F'!K54</f>
         <v>45.794</v>
       </c>
       <c r="G27" s="0"/>
       <c r="H27" s="0"/>
-      <c r="I27" s="90"/>
+      <c r="I27" s="97"/>
     </row>
     <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B28" s="86" t="s">
+      <c r="B28" s="93" t="s">
         <v>254</v>
       </c>
-      <c r="C28" s="82" t="n">
+      <c r="C28" s="89" t="n">
         <v>27.1</v>
       </c>
       <c r="D28" s="0"/>
-      <c r="E28" s="82" t="s">
+      <c r="E28" s="89" t="s">
         <v>254</v>
       </c>
-      <c r="F28" s="103" t="n">
+      <c r="F28" s="110" t="n">
         <f aca="false">'Modes A-F'!M54</f>
         <v>45.757</v>
       </c>
       <c r="G28" s="0"/>
       <c r="H28" s="0"/>
-      <c r="I28" s="90"/>
+      <c r="I28" s="97"/>
     </row>
     <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B29" s="86" t="s">
+      <c r="B29" s="93" t="s">
         <v>255</v>
       </c>
-      <c r="C29" s="82" t="n">
+      <c r="C29" s="89" t="n">
         <v>2.8</v>
       </c>
       <c r="D29" s="0"/>
-      <c r="E29" s="82" t="s">
+      <c r="E29" s="89" t="s">
         <v>255</v>
       </c>
-      <c r="F29" s="103" t="n">
+      <c r="F29" s="110" t="n">
         <f aca="false">'Modes A-F'!O54</f>
         <v>19.189</v>
       </c>
       <c r="G29" s="0"/>
       <c r="H29" s="0"/>
-      <c r="I29" s="90"/>
+      <c r="I29" s="97"/>
     </row>
     <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B30" s="86" t="s">
+      <c r="B30" s="93" t="s">
         <v>256</v>
       </c>
-      <c r="C30" s="82" t="n">
+      <c r="C30" s="89" t="n">
         <v>15</v>
       </c>
       <c r="D30" s="0"/>
-      <c r="E30" s="82" t="s">
+      <c r="E30" s="89" t="s">
         <v>256</v>
       </c>
-      <c r="F30" s="103" t="n">
+      <c r="F30" s="110" t="n">
         <f aca="false">'Modes A-F'!T54</f>
         <v>58.444</v>
       </c>
       <c r="G30" s="0"/>
       <c r="H30" s="0"/>
-      <c r="I30" s="90"/>
+      <c r="I30" s="97"/>
     </row>
     <row r="31" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B31" s="91" t="s">
+      <c r="B31" s="98" t="s">
         <v>248</v>
       </c>
-      <c r="C31" s="92" t="n">
+      <c r="C31" s="99" t="n">
         <v>55</v>
       </c>
-      <c r="D31" s="92"/>
-      <c r="E31" s="92"/>
-      <c r="F31" s="92"/>
-      <c r="G31" s="92"/>
-      <c r="H31" s="92"/>
-      <c r="I31" s="93"/>
+      <c r="D31" s="99"/>
+      <c r="E31" s="99"/>
+      <c r="F31" s="99"/>
+      <c r="G31" s="99"/>
+      <c r="H31" s="99"/>
+      <c r="I31" s="100"/>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -17169,7 +17226,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="B1:K7"/>
-  <sheetFormatPr defaultColWidth="11.82421875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.83984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="7.34"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="33"/>
@@ -17191,14 +17248,14 @@
       <c r="D1" s="14" t="s">
         <v>18</v>
       </c>
-      <c r="E1" s="104" t="s">
+      <c r="E1" s="111" t="s">
         <v>257</v>
       </c>
-      <c r="F1" s="104"/>
-      <c r="G1" s="105" t="s">
+      <c r="F1" s="111"/>
+      <c r="G1" s="112" t="s">
         <v>258</v>
       </c>
-      <c r="H1" s="105"/>
+      <c r="H1" s="112"/>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="44" t="s">
@@ -17224,25 +17281,25 @@
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B3" s="106" t="s">
+      <c r="B3" s="113" t="s">
         <v>92</v>
       </c>
-      <c r="C3" s="107" t="s">
+      <c r="C3" s="114" t="s">
         <v>93</v>
       </c>
-      <c r="D3" s="107" t="s">
+      <c r="D3" s="114" t="s">
         <v>259</v>
       </c>
-      <c r="E3" s="107" t="n">
+      <c r="E3" s="114" t="n">
         <v>8.77968</v>
       </c>
-      <c r="F3" s="107" t="n">
+      <c r="F3" s="114" t="n">
         <v>-2703</v>
       </c>
-      <c r="G3" s="108" t="n">
+      <c r="G3" s="115" t="n">
         <v>7.16226</v>
       </c>
-      <c r="H3" s="109" t="n">
+      <c r="H3" s="116" t="n">
         <v>-6620</v>
       </c>
     </row>
@@ -17305,11 +17362,11 @@
       <c r="G6" s="1" t="n">
         <v>15.99439325</v>
       </c>
-      <c r="I6" s="110" t="s">
+      <c r="I6" s="117" t="s">
         <v>262</v>
       </c>
-      <c r="J6" s="110"/>
-      <c r="K6" s="110"/>
+      <c r="J6" s="117"/>
+      <c r="K6" s="117"/>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D7" s="0" t="s">
@@ -17321,9 +17378,9 @@
       <c r="G7" s="1" t="n">
         <v>1.63763854</v>
       </c>
-      <c r="I7" s="110"/>
-      <c r="J7" s="110"/>
-      <c r="K7" s="110"/>
+      <c r="I7" s="117"/>
+      <c r="J7" s="117"/>
+      <c r="K7" s="117"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -17348,7 +17405,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:I36"/>
-  <sheetFormatPr defaultColWidth="11.82421875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.83984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="17.78"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="11.96"/>
@@ -17360,26 +17417,26 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="111"/>
-      <c r="B1" s="112"/>
-      <c r="C1" s="112"/>
-      <c r="D1" s="112"/>
-      <c r="E1" s="113" t="s">
+      <c r="A1" s="118"/>
+      <c r="B1" s="119"/>
+      <c r="C1" s="119"/>
+      <c r="D1" s="119"/>
+      <c r="E1" s="120" t="s">
         <v>264</v>
       </c>
-      <c r="F1" s="113" t="s">
+      <c r="F1" s="120" t="s">
         <v>6</v>
       </c>
-      <c r="G1" s="114" t="s">
+      <c r="G1" s="121" t="s">
         <v>265</v>
       </c>
-      <c r="H1" s="115" t="s">
+      <c r="H1" s="122" t="s">
         <v>266</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="116"/>
-      <c r="D2" s="117" t="s">
+      <c r="A2" s="123"/>
+      <c r="D2" s="124" t="s">
         <v>267</v>
       </c>
       <c r="E2" s="0" t="n">
@@ -17388,93 +17445,93 @@
       <c r="F2" s="0" t="n">
         <v>5</v>
       </c>
-      <c r="G2" s="118"/>
+      <c r="G2" s="125"/>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="119" t="s">
+      <c r="A3" s="126" t="s">
         <v>268</v>
       </c>
       <c r="B3" s="0" t="n">
         <v>9002</v>
       </c>
-      <c r="D3" s="117" t="s">
+      <c r="D3" s="124" t="s">
         <v>269</v>
       </c>
-      <c r="E3" s="120" t="n">
+      <c r="E3" s="127" t="n">
         <v>46.1092</v>
       </c>
-      <c r="F3" s="103" t="n">
+      <c r="F3" s="110" t="n">
         <f aca="false">E3-B3*TAN(2*(F2-E2)/1000)</f>
         <v>19.1031189817083</v>
       </c>
-      <c r="G3" s="121" t="n">
+      <c r="G3" s="128" t="n">
         <f aca="false">'Modes A-F'!O54</f>
         <v>19.189</v>
       </c>
-      <c r="H3" s="122" t="n">
+      <c r="H3" s="129" t="n">
         <f aca="false">G3-F3</f>
         <v>0.0858810182916656</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="119" t="s">
+      <c r="A4" s="126" t="s">
         <v>270</v>
       </c>
       <c r="B4" s="0" t="n">
         <f aca="false">B3+635</f>
         <v>9637</v>
       </c>
-      <c r="D4" s="117" t="s">
+      <c r="D4" s="124" t="s">
         <v>271</v>
       </c>
-      <c r="E4" s="103" t="n">
+      <c r="E4" s="110" t="n">
         <f aca="false">'Modes A-F'!K56</f>
         <v>127.868</v>
       </c>
-      <c r="F4" s="103" t="n">
+      <c r="F4" s="110" t="n">
         <f aca="false">E4-B4*TAN(2*(F2-E2)/1000)</f>
         <v>98.9569132666878</v>
       </c>
-      <c r="G4" s="121" t="n">
+      <c r="G4" s="128" t="n">
         <f aca="false">'Modes A-F'!O56</f>
         <v>99.085</v>
       </c>
-      <c r="H4" s="122" t="n">
+      <c r="H4" s="129" t="n">
         <f aca="false">G4-F4</f>
         <v>0.128086733312244</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="123" t="s">
+      <c r="A5" s="130" t="s">
         <v>272</v>
       </c>
-      <c r="B5" s="124" t="n">
+      <c r="B5" s="131" t="n">
         <f aca="false">B3+1790</f>
         <v>10792</v>
       </c>
-      <c r="C5" s="124"/>
-      <c r="D5" s="125" t="s">
+      <c r="C5" s="131"/>
+      <c r="D5" s="132" t="s">
         <v>273</v>
       </c>
-      <c r="E5" s="126" t="n">
+      <c r="E5" s="133" t="n">
         <f aca="false">'Modes A-F'!K57</f>
         <v>132.5</v>
       </c>
-      <c r="F5" s="126" t="n">
+      <c r="F5" s="133" t="n">
         <f aca="false">E5-B5*TAN(2*(F2-E2)/1000)</f>
         <v>100.12390287165</v>
       </c>
-      <c r="G5" s="127" t="n">
+      <c r="G5" s="134" t="n">
         <f aca="false">'Modes A-F'!O57</f>
         <v>100.567</v>
       </c>
-      <c r="H5" s="122" t="n">
+      <c r="H5" s="129" t="n">
         <f aca="false">G5-F5</f>
         <v>0.443097128349663</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H6" s="122" t="n">
+      <c r="H6" s="129" t="n">
         <f aca="false">AVERAGE(H3,H4,H5)</f>
         <v>0.219021626651191</v>
       </c>
@@ -17483,419 +17540,419 @@
       </c>
     </row>
     <row r="8" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="128" t="s">
+      <c r="A8" s="135" t="s">
         <v>1</v>
       </c>
-      <c r="B8" s="128"/>
-      <c r="C8" s="128"/>
-      <c r="D8" s="112"/>
-      <c r="E8" s="112"/>
-      <c r="F8" s="129" t="s">
+      <c r="B8" s="135"/>
+      <c r="C8" s="135"/>
+      <c r="D8" s="119"/>
+      <c r="E8" s="119"/>
+      <c r="F8" s="136" t="s">
         <v>275</v>
       </c>
-      <c r="G8" s="130" t="n">
+      <c r="G8" s="137" t="n">
         <v>-0.1</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="116"/>
-      <c r="D9" s="117" t="s">
+      <c r="A9" s="123"/>
+      <c r="D9" s="124" t="s">
         <v>267</v>
       </c>
       <c r="E9" s="0" t="n">
         <v>3.5</v>
       </c>
-      <c r="G9" s="118" t="n">
+      <c r="G9" s="125" t="n">
         <f aca="false">E9+G8</f>
         <v>3.4</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="119" t="s">
+      <c r="A10" s="126" t="s">
         <v>276</v>
       </c>
       <c r="B10" s="0" t="n">
         <v>10907</v>
       </c>
-      <c r="D10" s="117" t="s">
+      <c r="D10" s="124" t="s">
         <v>269</v>
       </c>
-      <c r="E10" s="122" t="n">
+      <c r="E10" s="129" t="n">
         <f aca="false">'Modes A-F'!E54</f>
         <v>37.717</v>
       </c>
-      <c r="F10" s="122"/>
-      <c r="G10" s="131" t="n">
+      <c r="F10" s="129"/>
+      <c r="G10" s="138" t="n">
         <f aca="false">E10-B10*TAN(2*(G9-E9)/1000)</f>
         <v>39.8984000290853</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="119" t="s">
+      <c r="A11" s="126" t="s">
         <v>277</v>
       </c>
       <c r="B11" s="0" t="n">
         <f aca="false">B10+635</f>
         <v>11542</v>
       </c>
-      <c r="D11" s="117" t="s">
+      <c r="D11" s="124" t="s">
         <v>271</v>
       </c>
-      <c r="E11" s="122" t="n">
+      <c r="E11" s="129" t="n">
         <f aca="false">'Modes A-F'!E57</f>
         <v>125.022</v>
       </c>
-      <c r="F11" s="122"/>
-      <c r="G11" s="131" t="n">
+      <c r="F11" s="129"/>
+      <c r="G11" s="138" t="n">
         <f aca="false">E11-B11*TAN(2*(G9-E9)/1000)</f>
         <v>127.330400030779</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="123" t="s">
+      <c r="A12" s="130" t="s">
         <v>278</v>
       </c>
-      <c r="B12" s="124" t="n">
+      <c r="B12" s="131" t="n">
         <f aca="false">B10+1790</f>
         <v>12697</v>
       </c>
-      <c r="C12" s="124"/>
-      <c r="D12" s="125" t="s">
+      <c r="C12" s="131"/>
+      <c r="D12" s="132" t="s">
         <v>273</v>
       </c>
-      <c r="E12" s="132" t="n">
+      <c r="E12" s="139" t="n">
         <f aca="false">'Modes A-F'!E58</f>
         <v>125.022</v>
       </c>
-      <c r="F12" s="132"/>
-      <c r="G12" s="133" t="n">
+      <c r="F12" s="139"/>
+      <c r="G12" s="140" t="n">
         <f aca="false">E12-B12*TAN(2*(G9-E9)/1000)</f>
         <v>127.561400033859</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="128" t="s">
+      <c r="A16" s="135" t="s">
         <v>3</v>
       </c>
-      <c r="B16" s="128"/>
-      <c r="C16" s="128"/>
-      <c r="D16" s="112"/>
-      <c r="E16" s="112"/>
-      <c r="F16" s="129" t="s">
+      <c r="B16" s="135"/>
+      <c r="C16" s="135"/>
+      <c r="D16" s="119"/>
+      <c r="E16" s="119"/>
+      <c r="F16" s="136" t="s">
         <v>275</v>
       </c>
-      <c r="G16" s="112" t="n">
+      <c r="G16" s="119" t="n">
         <v>0.275</v>
       </c>
-      <c r="H16" s="112"/>
-      <c r="I16" s="130"/>
+      <c r="H16" s="119"/>
+      <c r="I16" s="137"/>
     </row>
     <row r="17" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="116"/>
-      <c r="D17" s="117" t="s">
+      <c r="A17" s="123"/>
+      <c r="D17" s="124" t="s">
         <v>267</v>
       </c>
       <c r="E17" s="0" t="n">
         <v>3.225</v>
       </c>
-      <c r="G17" s="71" t="n">
+      <c r="G17" s="78" t="n">
         <f aca="false">E17+G16</f>
         <v>3.5</v>
       </c>
       <c r="H17" s="60" t="s">
         <v>279</v>
       </c>
-      <c r="I17" s="118" t="n">
+      <c r="I17" s="125" t="n">
         <f aca="false">B18*TAN(2*(E9-G17)/1000)</f>
         <v>0</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="119" t="s">
+      <c r="A18" s="126" t="s">
         <v>280</v>
       </c>
       <c r="B18" s="0" t="n">
         <v>1908</v>
       </c>
-      <c r="D18" s="117" t="s">
+      <c r="D18" s="124" t="s">
         <v>281</v>
       </c>
       <c r="E18" s="0" t="n">
         <v>-7.25</v>
       </c>
-      <c r="G18" s="134" t="n">
+      <c r="G18" s="141" t="n">
         <f aca="false">E18+B18*TAN(2*(G17-E17)/1000)</f>
         <v>-6.20059989418549</v>
       </c>
-      <c r="I18" s="118"/>
+      <c r="I18" s="125"/>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="116"/>
-      <c r="D19" s="117" t="s">
+      <c r="A19" s="123"/>
+      <c r="D19" s="124" t="s">
         <v>282</v>
       </c>
       <c r="E19" s="0" t="n">
         <f aca="false">3.5 + (3.5-E17)</f>
         <v>3.775</v>
       </c>
-      <c r="G19" s="71" t="n">
+      <c r="G19" s="78" t="n">
         <f aca="false">E19-G16</f>
         <v>3.5</v>
       </c>
-      <c r="I19" s="118"/>
+      <c r="I19" s="125"/>
     </row>
     <row r="20" customFormat="false" ht="23.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="116"/>
-      <c r="D20" s="117"/>
-      <c r="G20" s="135" t="s">
+      <c r="A20" s="123"/>
+      <c r="D20" s="124"/>
+      <c r="G20" s="142" t="s">
         <v>283</v>
       </c>
-      <c r="I20" s="118"/>
+      <c r="I20" s="125"/>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="116"/>
-      <c r="F21" s="136" t="s">
+      <c r="A21" s="123"/>
+      <c r="F21" s="143" t="s">
         <v>265</v>
       </c>
-      <c r="I21" s="118"/>
+      <c r="I21" s="125"/>
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="119" t="s">
+      <c r="A22" s="126" t="s">
         <v>268</v>
       </c>
       <c r="B22" s="0" t="n">
         <v>9002</v>
       </c>
-      <c r="D22" s="117" t="s">
+      <c r="D22" s="124" t="s">
         <v>269</v>
       </c>
-      <c r="E22" s="122" t="n">
+      <c r="E22" s="129" t="n">
         <f aca="false">E10-B22*TAN(2*(E19)/1000)+I17</f>
         <v>-30.2493914229833</v>
       </c>
-      <c r="F22" s="137" t="n">
+      <c r="F22" s="144" t="n">
         <f aca="false">'Modes A-F'!I54</f>
         <v>-23.201</v>
       </c>
-      <c r="G22" s="122" t="n">
+      <c r="G22" s="129" t="n">
         <f aca="false">E10-B22*TAN(2*(G19)/1000)+I17</f>
         <v>-25.29802924884</v>
       </c>
-      <c r="I22" s="118"/>
+      <c r="I22" s="125"/>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="119" t="s">
+      <c r="A23" s="126" t="s">
         <v>270</v>
       </c>
       <c r="B23" s="0" t="n">
         <f aca="false">B22+635</f>
         <v>9637</v>
       </c>
-      <c r="D23" s="117" t="s">
+      <c r="D23" s="124" t="s">
         <v>271</v>
       </c>
-      <c r="E23" s="122" t="n">
+      <c r="E23" s="129" t="n">
         <f aca="false">E11-B23*TAN(2*(E19)/1000)+I17</f>
         <v>52.2612674801944</v>
       </c>
-      <c r="F23" s="137" t="n">
+      <c r="F23" s="144" t="n">
         <f aca="false">'Modes A-F'!I56</f>
         <v>54.064</v>
       </c>
-      <c r="G23" s="122" t="n">
+      <c r="G23" s="129" t="n">
         <f aca="false">E11-B23*TAN(2*(G19)/1000)+I17</f>
         <v>57.5618981480704</v>
       </c>
-      <c r="I23" s="118"/>
+      <c r="I23" s="125"/>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="123" t="s">
+      <c r="A24" s="130" t="s">
         <v>272</v>
       </c>
-      <c r="B24" s="124" t="n">
+      <c r="B24" s="131" t="n">
         <f aca="false">B22+1790</f>
         <v>10792</v>
       </c>
-      <c r="C24" s="124"/>
-      <c r="D24" s="125" t="s">
+      <c r="C24" s="131"/>
+      <c r="D24" s="132" t="s">
         <v>273</v>
       </c>
-      <c r="E24" s="132" t="n">
+      <c r="E24" s="139" t="n">
         <f aca="false">E12-B24*TAN(2*(E19)/1000)+I17</f>
         <v>43.5408517843995</v>
       </c>
-      <c r="F24" s="138" t="n">
+      <c r="F24" s="145" t="n">
         <f aca="false">'Modes A-F'!I57</f>
         <v>51.187</v>
       </c>
-      <c r="G24" s="139" t="n">
+      <c r="G24" s="146" t="n">
         <f aca="false">E12-B24*TAN(2*(G19)/1000)+I17</f>
         <v>49.476766090482</v>
       </c>
-      <c r="H24" s="124"/>
-      <c r="I24" s="140"/>
+      <c r="H24" s="131"/>
+      <c r="I24" s="147"/>
     </row>
     <row r="28" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="141" t="s">
+      <c r="A28" s="148" t="s">
         <v>2</v>
       </c>
-      <c r="B28" s="141"/>
-      <c r="C28" s="141"/>
-      <c r="D28" s="112"/>
-      <c r="E28" s="112"/>
-      <c r="F28" s="129" t="s">
+      <c r="B28" s="148"/>
+      <c r="C28" s="148"/>
+      <c r="D28" s="119"/>
+      <c r="E28" s="119"/>
+      <c r="F28" s="136" t="s">
         <v>275</v>
       </c>
-      <c r="G28" s="112" t="n">
+      <c r="G28" s="119" t="n">
         <v>0.275</v>
       </c>
-      <c r="H28" s="112"/>
-      <c r="I28" s="130"/>
+      <c r="H28" s="119"/>
+      <c r="I28" s="137"/>
     </row>
     <row r="29" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="116"/>
-      <c r="D29" s="117" t="s">
+      <c r="A29" s="123"/>
+      <c r="D29" s="124" t="s">
         <v>267</v>
       </c>
       <c r="E29" s="0" t="n">
         <v>3.225</v>
       </c>
-      <c r="G29" s="71" t="n">
+      <c r="G29" s="78" t="n">
         <f aca="false">E29+G28</f>
         <v>3.5</v>
       </c>
       <c r="H29" s="60" t="s">
         <v>279</v>
       </c>
-      <c r="I29" s="118" t="n">
+      <c r="I29" s="125" t="n">
         <f aca="false">B30*TAN(2*(E9-G29)/1000)</f>
         <v>0</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="119" t="s">
+      <c r="A30" s="126" t="s">
         <v>280</v>
       </c>
       <c r="B30" s="0" t="n">
         <v>1908</v>
       </c>
-      <c r="D30" s="117" t="s">
+      <c r="D30" s="124" t="s">
         <v>281</v>
       </c>
       <c r="E30" s="0" t="n">
         <v>-6.583</v>
       </c>
-      <c r="G30" s="134" t="n">
+      <c r="G30" s="141" t="n">
         <f aca="false">E30+B30*TAN(2*(G29-E29)/1000)</f>
         <v>-5.53359989418549</v>
       </c>
-      <c r="I30" s="118"/>
+      <c r="I30" s="125"/>
     </row>
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="116"/>
-      <c r="D31" s="117" t="s">
+      <c r="A31" s="123"/>
+      <c r="D31" s="124" t="s">
         <v>282</v>
       </c>
       <c r="E31" s="0" t="n">
         <f aca="false">5+(3.5-E29)</f>
         <v>5.275</v>
       </c>
-      <c r="G31" s="71" t="n">
+      <c r="G31" s="78" t="n">
         <f aca="false">E31-G28</f>
         <v>5</v>
       </c>
-      <c r="I31" s="118"/>
+      <c r="I31" s="125"/>
     </row>
     <row r="32" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="116"/>
-      <c r="D32" s="117"/>
-      <c r="G32" s="135" t="s">
+      <c r="A32" s="123"/>
+      <c r="D32" s="124"/>
+      <c r="G32" s="142" t="s">
         <v>283</v>
       </c>
-      <c r="I32" s="118"/>
+      <c r="I32" s="125"/>
     </row>
     <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="116"/>
-      <c r="F33" s="136" t="s">
+      <c r="A33" s="123"/>
+      <c r="F33" s="143" t="s">
         <v>265</v>
       </c>
-      <c r="I33" s="118"/>
+      <c r="I33" s="125"/>
     </row>
     <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="119" t="s">
+      <c r="A34" s="126" t="s">
         <v>268</v>
       </c>
       <c r="B34" s="0" t="n">
         <v>9002</v>
       </c>
-      <c r="D34" s="117" t="s">
+      <c r="D34" s="124" t="s">
         <v>269</v>
       </c>
-      <c r="E34" s="122" t="n">
+      <c r="E34" s="129" t="n">
         <f aca="false">E10-B34*TAN(2*(E31)/1000)</f>
         <v>-57.2576236638297</v>
       </c>
-      <c r="F34" s="137" t="n">
+      <c r="F34" s="144" t="n">
         <f aca="false">'Modes A-F'!G54</f>
         <v>-55.188</v>
       </c>
-      <c r="G34" s="122" t="n">
+      <c r="G34" s="129" t="n">
         <f aca="false">E10-B34*TAN(2*(G31)/1000)+I29</f>
         <v>-52.3060007866982</v>
       </c>
-      <c r="I34" s="118"/>
+      <c r="I34" s="125"/>
     </row>
     <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="119" t="s">
+      <c r="A35" s="126" t="s">
         <v>270</v>
       </c>
       <c r="B35" s="0" t="n">
         <f aca="false">B34+635</f>
         <v>9637</v>
       </c>
-      <c r="D35" s="117" t="s">
+      <c r="D35" s="124" t="s">
         <v>271</v>
       </c>
-      <c r="E35" s="122" t="n">
+      <c r="E35" s="129" t="n">
         <f aca="false">E11-B35*TAN(2*(E31)/1000)</f>
         <v>23.3478777773465</v>
       </c>
-      <c r="F35" s="137" t="n">
+      <c r="F35" s="144" t="n">
         <f aca="false">'Modes A-F'!G56</f>
         <v>24.4104</v>
       </c>
-      <c r="G35" s="122" t="n">
+      <c r="G35" s="129" t="n">
         <f aca="false">E11-B35*TAN(2*(G31)/1000)+I29</f>
         <v>28.6487875381681</v>
       </c>
-      <c r="I35" s="118"/>
+      <c r="I35" s="125"/>
     </row>
     <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="123" t="s">
+      <c r="A36" s="130" t="s">
         <v>272</v>
       </c>
-      <c r="B36" s="124" t="n">
+      <c r="B36" s="131" t="n">
         <f aca="false">B34+1790</f>
         <v>10792</v>
       </c>
-      <c r="C36" s="124"/>
-      <c r="D36" s="125" t="s">
+      <c r="C36" s="131"/>
+      <c r="D36" s="132" t="s">
         <v>273</v>
       </c>
-      <c r="E36" s="132" t="n">
+      <c r="E36" s="139" t="n">
         <f aca="false">E12-B36*TAN(2*(E31)/1000)</f>
         <v>11.162175674289</v>
       </c>
-      <c r="F36" s="138" t="n">
+      <c r="F36" s="145" t="n">
         <f aca="false">'Modes A-F'!G57</f>
         <v>12.81</v>
       </c>
-      <c r="G36" s="132" t="n">
+      <c r="G36" s="139" t="n">
         <f aca="false">E12-B36*TAN(2*(G31)/1000)+I29</f>
         <v>17.0984025227675</v>
       </c>
-      <c r="H36" s="124"/>
-      <c r="I36" s="140"/>
+      <c r="H36" s="131"/>
+      <c r="I36" s="147"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -17919,7 +17976,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:CX484"/>
-  <sheetFormatPr defaultColWidth="11.82421875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.83984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="35.26"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="102" min="2" style="0" width="11.96"/>
@@ -17993,7 +18050,7 @@
       <c r="A9" s="0" t="s">
         <v>292</v>
       </c>
-      <c r="B9" s="142" t="n">
+      <c r="B9" s="149" t="n">
         <v>1E-006</v>
       </c>
     </row>
@@ -18017,7 +18074,7 @@
       <c r="A12" s="0" t="s">
         <v>295</v>
       </c>
-      <c r="B12" s="142" t="n">
+      <c r="B12" s="149" t="n">
         <v>1E-005</v>
       </c>
     </row>
@@ -18113,7 +18170,7 @@
       <c r="A24" s="0" t="s">
         <v>307</v>
       </c>
-      <c r="B24" s="142" t="n">
+      <c r="B24" s="149" t="n">
         <v>1E-006</v>
       </c>
     </row>
@@ -18137,7 +18194,7 @@
       <c r="A27" s="0" t="s">
         <v>310</v>
       </c>
-      <c r="B27" s="142" t="n">
+      <c r="B27" s="149" t="n">
         <v>1E-005</v>
       </c>
     </row>
@@ -18233,7 +18290,7 @@
       <c r="A39" s="0" t="s">
         <v>322</v>
       </c>
-      <c r="B39" s="142" t="n">
+      <c r="B39" s="149" t="n">
         <v>1E-006</v>
       </c>
     </row>
@@ -18257,7 +18314,7 @@
       <c r="A42" s="0" t="s">
         <v>325</v>
       </c>
-      <c r="B42" s="142" t="n">
+      <c r="B42" s="149" t="n">
         <v>1E-005</v>
       </c>
     </row>
@@ -18353,7 +18410,7 @@
       <c r="A54" s="0" t="s">
         <v>337</v>
       </c>
-      <c r="B54" s="142" t="n">
+      <c r="B54" s="149" t="n">
         <v>1E-006</v>
       </c>
     </row>
@@ -18377,7 +18434,7 @@
       <c r="A57" s="0" t="s">
         <v>340</v>
       </c>
-      <c r="B57" s="142" t="n">
+      <c r="B57" s="149" t="n">
         <v>1E-005</v>
       </c>
     </row>
@@ -18441,7 +18498,7 @@
       <c r="A65" s="0" t="s">
         <v>348</v>
       </c>
-      <c r="B65" s="142" t="n">
+      <c r="B65" s="149" t="n">
         <v>8.1921E-011</v>
       </c>
     </row>
@@ -18449,7 +18506,7 @@
       <c r="A66" s="0" t="s">
         <v>349</v>
       </c>
-      <c r="B66" s="142" t="n">
+      <c r="B66" s="149" t="n">
         <v>6.1817E-009</v>
       </c>
     </row>
@@ -18457,7 +18514,7 @@
       <c r="A67" s="0" t="s">
         <v>350</v>
       </c>
-      <c r="B67" s="142" t="n">
+      <c r="B67" s="149" t="n">
         <v>-8.139E-009</v>
       </c>
     </row>
@@ -18465,7 +18522,7 @@
       <c r="A68" s="0" t="s">
         <v>351</v>
       </c>
-      <c r="B68" s="142" t="n">
+      <c r="B68" s="149" t="n">
         <v>4.2612E-009</v>
       </c>
     </row>
@@ -18785,7 +18842,7 @@
       <c r="A108" s="0" t="s">
         <v>391</v>
       </c>
-      <c r="B108" s="142" t="n">
+      <c r="B108" s="149" t="n">
         <v>1E-006</v>
       </c>
     </row>
@@ -18809,7 +18866,7 @@
       <c r="A111" s="0" t="s">
         <v>394</v>
       </c>
-      <c r="B111" s="142" t="n">
+      <c r="B111" s="149" t="n">
         <v>1E-005</v>
       </c>
     </row>
@@ -18905,7 +18962,7 @@
       <c r="A123" s="0" t="s">
         <v>406</v>
       </c>
-      <c r="B123" s="142" t="n">
+      <c r="B123" s="149" t="n">
         <v>1E-006</v>
       </c>
     </row>
@@ -18929,7 +18986,7 @@
       <c r="A126" s="0" t="s">
         <v>409</v>
       </c>
-      <c r="B126" s="142" t="n">
+      <c r="B126" s="149" t="n">
         <v>1E-005</v>
       </c>
     </row>
@@ -19025,7 +19082,7 @@
       <c r="A138" s="0" t="s">
         <v>421</v>
       </c>
-      <c r="B138" s="142" t="n">
+      <c r="B138" s="149" t="n">
         <v>1E-006</v>
       </c>
     </row>
@@ -19049,7 +19106,7 @@
       <c r="A141" s="0" t="s">
         <v>424</v>
       </c>
-      <c r="B141" s="142" t="n">
+      <c r="B141" s="149" t="n">
         <v>1E-005</v>
       </c>
     </row>
@@ -19145,7 +19202,7 @@
       <c r="A153" s="0" t="s">
         <v>436</v>
       </c>
-      <c r="B153" s="142" t="n">
+      <c r="B153" s="149" t="n">
         <v>1E-006</v>
       </c>
     </row>
@@ -19169,7 +19226,7 @@
       <c r="A156" s="0" t="s">
         <v>439</v>
       </c>
-      <c r="B156" s="142" t="n">
+      <c r="B156" s="149" t="n">
         <v>1E-005</v>
       </c>
     </row>
@@ -19233,7 +19290,7 @@
       <c r="A164" s="0" t="s">
         <v>447</v>
       </c>
-      <c r="B164" s="142" t="n">
+      <c r="B164" s="149" t="n">
         <v>1.9024E-008</v>
       </c>
     </row>
@@ -19241,7 +19298,7 @@
       <c r="A165" s="0" t="s">
         <v>448</v>
       </c>
-      <c r="B165" s="142" t="n">
+      <c r="B165" s="149" t="n">
         <v>-9.5679E-009</v>
       </c>
     </row>
@@ -19249,7 +19306,7 @@
       <c r="A166" s="0" t="s">
         <v>449</v>
       </c>
-      <c r="B166" s="142" t="n">
+      <c r="B166" s="149" t="n">
         <v>-1.1631E-009</v>
       </c>
     </row>
@@ -19257,7 +19314,7 @@
       <c r="A167" s="0" t="s">
         <v>450</v>
       </c>
-      <c r="B167" s="142" t="n">
+      <c r="B167" s="149" t="n">
         <v>1.027E-008</v>
       </c>
     </row>
@@ -19393,7 +19450,7 @@
       <c r="A184" s="0" t="s">
         <v>467</v>
       </c>
-      <c r="B184" s="142" t="n">
+      <c r="B184" s="149" t="n">
         <v>2.8833E-008</v>
       </c>
     </row>
@@ -19401,7 +19458,7 @@
       <c r="A185" s="0" t="s">
         <v>468</v>
       </c>
-      <c r="B185" s="142" t="n">
+      <c r="B185" s="149" t="n">
         <v>2.8833E-008</v>
       </c>
     </row>
@@ -19433,7 +19490,7 @@
       <c r="A189" s="0" t="s">
         <v>472</v>
       </c>
-      <c r="B189" s="142" t="n">
+      <c r="B189" s="149" t="n">
         <v>4761600</v>
       </c>
     </row>
@@ -19457,7 +19514,7 @@
       <c r="A192" s="0" t="s">
         <v>475</v>
       </c>
-      <c r="B192" s="142" t="n">
+      <c r="B192" s="149" t="n">
         <v>2.8343E-008</v>
       </c>
     </row>
@@ -19465,7 +19522,7 @@
       <c r="A193" s="0" t="s">
         <v>476</v>
       </c>
-      <c r="B193" s="142" t="n">
+      <c r="B193" s="149" t="n">
         <v>-7.401E-010</v>
       </c>
     </row>
@@ -19473,7 +19530,7 @@
       <c r="A194" s="0" t="s">
         <v>477</v>
       </c>
-      <c r="B194" s="142" t="n">
+      <c r="B194" s="149" t="n">
         <v>-1.4084E-009</v>
       </c>
     </row>
@@ -19481,7 +19538,7 @@
       <c r="A195" s="0" t="s">
         <v>478</v>
       </c>
-      <c r="B195" s="142" t="n">
+      <c r="B195" s="149" t="n">
         <v>2.0325E-008</v>
       </c>
     </row>
@@ -20905,40 +20962,40 @@
       <c r="B337" s="0" t="n">
         <v>12</v>
       </c>
-      <c r="C337" s="142" t="n">
+      <c r="C337" s="149" t="n">
         <v>8.3006E-011</v>
       </c>
-      <c r="D337" s="142" t="n">
+      <c r="D337" s="149" t="n">
         <v>8.2839E-011</v>
       </c>
-      <c r="E337" s="142" t="n">
+      <c r="E337" s="149" t="n">
         <v>8.2777E-011</v>
       </c>
-      <c r="F337" s="142" t="n">
+      <c r="F337" s="149" t="n">
         <v>8.1528E-011</v>
       </c>
-      <c r="G337" s="142" t="n">
+      <c r="G337" s="149" t="n">
         <v>8.2662E-011</v>
       </c>
-      <c r="H337" s="142" t="n">
+      <c r="H337" s="149" t="n">
         <v>8.3572E-011</v>
       </c>
-      <c r="I337" s="142" t="n">
+      <c r="I337" s="149" t="n">
         <v>8.489E-011</v>
       </c>
-      <c r="J337" s="142" t="n">
+      <c r="J337" s="149" t="n">
         <v>8.3896E-011</v>
       </c>
-      <c r="K337" s="142" t="n">
+      <c r="K337" s="149" t="n">
         <v>8.2012E-011</v>
       </c>
-      <c r="L337" s="142" t="n">
+      <c r="L337" s="149" t="n">
         <v>8.0897E-011</v>
       </c>
-      <c r="M337" s="142" t="n">
+      <c r="M337" s="149" t="n">
         <v>8.29E-011</v>
       </c>
-      <c r="N337" s="142" t="n">
+      <c r="N337" s="149" t="n">
         <v>8.0797E-011</v>
       </c>
     </row>
@@ -20949,40 +21006,40 @@
       <c r="B338" s="0" t="n">
         <v>12</v>
       </c>
-      <c r="C338" s="142" t="n">
+      <c r="C338" s="149" t="n">
         <v>6.3068E-009</v>
       </c>
-      <c r="D338" s="142" t="n">
+      <c r="D338" s="149" t="n">
         <v>6.0737E-009</v>
       </c>
-      <c r="E338" s="142" t="n">
+      <c r="E338" s="149" t="n">
         <v>6.6921E-009</v>
       </c>
-      <c r="F338" s="142" t="n">
+      <c r="F338" s="149" t="n">
         <v>5.7007E-009</v>
       </c>
-      <c r="G338" s="142" t="n">
+      <c r="G338" s="149" t="n">
         <v>5.6393E-009</v>
       </c>
-      <c r="H338" s="142" t="n">
+      <c r="H338" s="149" t="n">
         <v>6.6627E-009</v>
       </c>
-      <c r="I338" s="142" t="n">
+      <c r="I338" s="149" t="n">
         <v>6.6038E-009</v>
       </c>
-      <c r="J338" s="142" t="n">
+      <c r="J338" s="149" t="n">
         <v>5.87E-009</v>
       </c>
-      <c r="K338" s="142" t="n">
+      <c r="K338" s="149" t="n">
         <v>6.1792E-009</v>
       </c>
-      <c r="L338" s="142" t="n">
+      <c r="L338" s="149" t="n">
         <v>5.3276E-009</v>
       </c>
-      <c r="M338" s="142" t="n">
+      <c r="M338" s="149" t="n">
         <v>6.513E-009</v>
       </c>
-      <c r="N338" s="142" t="n">
+      <c r="N338" s="149" t="n">
         <v>5.9829E-009</v>
       </c>
     </row>
@@ -20993,40 +21050,40 @@
       <c r="B339" s="0" t="n">
         <v>12</v>
       </c>
-      <c r="C339" s="142" t="n">
+      <c r="C339" s="149" t="n">
         <v>-7.2948E-009</v>
       </c>
-      <c r="D339" s="142" t="n">
+      <c r="D339" s="149" t="n">
         <v>-7.6015E-009</v>
       </c>
-      <c r="E339" s="142" t="n">
+      <c r="E339" s="149" t="n">
         <v>-7.4862E-009</v>
       </c>
-      <c r="F339" s="142" t="n">
+      <c r="F339" s="149" t="n">
         <v>-8.5513E-009</v>
       </c>
-      <c r="G339" s="142" t="n">
+      <c r="G339" s="149" t="n">
         <v>-8.3206E-009</v>
       </c>
-      <c r="H339" s="142" t="n">
+      <c r="H339" s="149" t="n">
         <v>-7.5942E-009</v>
       </c>
-      <c r="I339" s="142" t="n">
+      <c r="I339" s="149" t="n">
         <v>-7.5377E-009</v>
       </c>
-      <c r="J339" s="142" t="n">
+      <c r="J339" s="149" t="n">
         <v>-8.5415E-009</v>
       </c>
-      <c r="K339" s="142" t="n">
+      <c r="K339" s="149" t="n">
         <v>-7.7635E-009</v>
       </c>
-      <c r="L339" s="142" t="n">
+      <c r="L339" s="149" t="n">
         <v>-8.0482E-009</v>
       </c>
-      <c r="M339" s="142" t="n">
+      <c r="M339" s="149" t="n">
         <v>-8.2175E-009</v>
       </c>
-      <c r="N339" s="142" t="n">
+      <c r="N339" s="149" t="n">
         <v>-7.9966E-009</v>
       </c>
     </row>
@@ -21037,40 +21094,40 @@
       <c r="B340" s="0" t="n">
         <v>12</v>
       </c>
-      <c r="C340" s="142" t="n">
+      <c r="C340" s="149" t="n">
         <v>4.8625E-009</v>
       </c>
-      <c r="D340" s="142" t="n">
+      <c r="D340" s="149" t="n">
         <v>4.433E-009</v>
       </c>
-      <c r="E340" s="142" t="n">
+      <c r="E340" s="149" t="n">
         <v>3.4611E-009</v>
       </c>
-      <c r="F340" s="142" t="n">
+      <c r="F340" s="149" t="n">
         <v>3.9372E-009</v>
       </c>
-      <c r="G340" s="142" t="n">
+      <c r="G340" s="149" t="n">
         <v>4.8526E-009</v>
       </c>
-      <c r="H340" s="142" t="n">
+      <c r="H340" s="149" t="n">
         <v>4.5041E-009</v>
       </c>
-      <c r="I340" s="142" t="n">
+      <c r="I340" s="149" t="n">
         <v>4.5311E-009</v>
       </c>
-      <c r="J340" s="142" t="n">
+      <c r="J340" s="149" t="n">
         <v>4.2882E-009</v>
       </c>
-      <c r="K340" s="142" t="n">
+      <c r="K340" s="149" t="n">
         <v>4.4551E-009</v>
       </c>
-      <c r="L340" s="142" t="n">
+      <c r="L340" s="149" t="n">
         <v>4.136E-009</v>
       </c>
-      <c r="M340" s="142" t="n">
+      <c r="M340" s="149" t="n">
         <v>3.9078E-009</v>
       </c>
-      <c r="N340" s="142" t="n">
+      <c r="N340" s="149" t="n">
         <v>3.9593E-009</v>
       </c>
     </row>
@@ -21785,40 +21842,40 @@
       <c r="B357" s="0" t="n">
         <v>12</v>
       </c>
-      <c r="C357" s="142" t="n">
+      <c r="C357" s="149" t="n">
         <v>2.1231E-008</v>
       </c>
-      <c r="D357" s="142" t="n">
+      <c r="D357" s="149" t="n">
         <v>1.9514E-008</v>
       </c>
-      <c r="E357" s="142" t="n">
+      <c r="E357" s="149" t="n">
         <v>1.8533E-008</v>
       </c>
-      <c r="F357" s="142" t="n">
+      <c r="F357" s="149" t="n">
         <v>2.1231E-008</v>
       </c>
-      <c r="G357" s="142" t="n">
+      <c r="G357" s="149" t="n">
         <v>2.4174E-008</v>
       </c>
-      <c r="H357" s="142" t="n">
+      <c r="H357" s="149" t="n">
         <v>1.9024E-008</v>
       </c>
-      <c r="I357" s="142" t="n">
+      <c r="I357" s="149" t="n">
         <v>2.8588E-008</v>
       </c>
-      <c r="J357" s="142" t="n">
+      <c r="J357" s="149" t="n">
         <v>1.9024E-008</v>
       </c>
-      <c r="K357" s="142" t="n">
+      <c r="K357" s="149" t="n">
         <v>3.2757E-008</v>
       </c>
-      <c r="L357" s="142" t="n">
+      <c r="L357" s="149" t="n">
         <v>3.5455E-008</v>
       </c>
-      <c r="M357" s="142" t="n">
+      <c r="M357" s="149" t="n">
         <v>2.025E-008</v>
       </c>
-      <c r="N357" s="142" t="n">
+      <c r="N357" s="149" t="n">
         <v>2.1231E-008</v>
       </c>
     </row>
@@ -21829,40 +21886,40 @@
       <c r="B358" s="0" t="n">
         <v>12</v>
       </c>
-      <c r="C358" s="142" t="n">
+      <c r="C358" s="149" t="n">
         <v>-1.766E-008</v>
       </c>
-      <c r="D358" s="142" t="n">
+      <c r="D358" s="149" t="n">
         <v>-4.4184E-009</v>
       </c>
-      <c r="E358" s="142" t="n">
+      <c r="E358" s="149" t="n">
         <v>-1.1284E-008</v>
       </c>
-      <c r="F358" s="142" t="n">
+      <c r="F358" s="149" t="n">
         <v>-1.1039E-008</v>
       </c>
-      <c r="G358" s="142" t="n">
+      <c r="G358" s="149" t="n">
         <v>-9.5679E-009</v>
       </c>
-      <c r="H358" s="142" t="n">
+      <c r="H358" s="149" t="n">
         <v>-1.1284E-008</v>
       </c>
-      <c r="I358" s="142" t="n">
+      <c r="I358" s="149" t="n">
         <v>-2.2114E-009</v>
       </c>
-      <c r="J358" s="142" t="n">
+      <c r="J358" s="149" t="n">
         <v>-5.3992E-009</v>
       </c>
-      <c r="K358" s="142" t="n">
+      <c r="K358" s="149" t="n">
         <v>9.7642E-010</v>
       </c>
-      <c r="L358" s="142" t="n">
+      <c r="L358" s="149" t="n">
         <v>6.3712E-009</v>
       </c>
-      <c r="M358" s="142" t="n">
+      <c r="M358" s="149" t="n">
         <v>-1.153E-008</v>
       </c>
-      <c r="N358" s="142" t="n">
+      <c r="N358" s="149" t="n">
         <v>-9.8131E-009</v>
       </c>
     </row>
@@ -21873,40 +21930,40 @@
       <c r="B359" s="0" t="n">
         <v>12</v>
       </c>
-      <c r="C359" s="142" t="n">
+      <c r="C359" s="149" t="n">
         <v>-9.0112E-009</v>
       </c>
-      <c r="D359" s="142" t="n">
+      <c r="D359" s="149" t="n">
         <v>-4.3514E-009</v>
       </c>
-      <c r="E359" s="142" t="n">
+      <c r="E359" s="149" t="n">
         <v>-6.0682E-009</v>
       </c>
-      <c r="F359" s="142" t="n">
+      <c r="F359" s="149" t="n">
         <v>-9.0112E-009</v>
       </c>
-      <c r="G359" s="142" t="n">
+      <c r="G359" s="149" t="n">
         <v>-4.5967E-009</v>
       </c>
-      <c r="H359" s="142" t="n">
+      <c r="H359" s="149" t="n">
         <v>-1.0483E-008</v>
       </c>
-      <c r="I359" s="142" t="n">
+      <c r="I359" s="149" t="n">
         <v>7.6659E-009</v>
       </c>
-      <c r="J359" s="142" t="n">
+      <c r="J359" s="149" t="n">
         <v>-3.3704E-009</v>
       </c>
-      <c r="K359" s="142" t="n">
+      <c r="K359" s="149" t="n">
         <v>6.6849E-009</v>
       </c>
-      <c r="L359" s="142" t="n">
+      <c r="L359" s="149" t="n">
         <v>5.2134E-009</v>
       </c>
-      <c r="M359" s="142" t="n">
+      <c r="M359" s="149" t="n">
         <v>-1.6536E-009</v>
       </c>
-      <c r="N359" s="142" t="n">
+      <c r="N359" s="149" t="n">
         <v>-5.5777E-009</v>
       </c>
     </row>
@@ -21917,40 +21974,40 @@
       <c r="B360" s="0" t="n">
         <v>12</v>
       </c>
-      <c r="C360" s="142" t="n">
+      <c r="C360" s="149" t="n">
         <v>7.8174E-009</v>
       </c>
-      <c r="D360" s="142" t="n">
+      <c r="D360" s="149" t="n">
         <v>2.3513E-008</v>
       </c>
-      <c r="E360" s="142" t="n">
+      <c r="E360" s="149" t="n">
         <v>1.7382E-008</v>
       </c>
-      <c r="F360" s="142" t="n">
+      <c r="F360" s="149" t="n">
         <v>1.1006E-008</v>
       </c>
-      <c r="G360" s="142" t="n">
+      <c r="G360" s="149" t="n">
         <v>1.5665E-008</v>
       </c>
-      <c r="H360" s="142" t="n">
+      <c r="H360" s="149" t="n">
         <v>1.2477E-008</v>
       </c>
-      <c r="I360" s="142" t="n">
+      <c r="I360" s="149" t="n">
         <v>2.057E-008</v>
       </c>
-      <c r="J360" s="142" t="n">
+      <c r="J360" s="149" t="n">
         <v>1.9835E-008</v>
       </c>
-      <c r="K360" s="142" t="n">
+      <c r="K360" s="149" t="n">
         <v>2.5721E-008</v>
       </c>
-      <c r="L360" s="142" t="n">
+      <c r="L360" s="149" t="n">
         <v>2.5475E-008</v>
       </c>
-      <c r="M360" s="142" t="n">
+      <c r="M360" s="149" t="n">
         <v>1.076E-008</v>
       </c>
-      <c r="N360" s="142" t="n">
+      <c r="N360" s="149" t="n">
         <v>1.3213E-008</v>
       </c>
     </row>
@@ -22093,7 +22150,7 @@
       <c r="B364" s="0" t="n">
         <v>12</v>
       </c>
-      <c r="C364" s="142" t="n">
+      <c r="C364" s="149" t="n">
         <v>2.8343E-008</v>
       </c>
       <c r="D364" s="0" t="n">
@@ -22137,7 +22194,7 @@
       <c r="B365" s="0" t="n">
         <v>12</v>
       </c>
-      <c r="C365" s="142" t="n">
+      <c r="C365" s="149" t="n">
         <v>-7.401E-010</v>
       </c>
       <c r="D365" s="0" t="n">
@@ -22181,7 +22238,7 @@
       <c r="B366" s="0" t="n">
         <v>12</v>
       </c>
-      <c r="C366" s="142" t="n">
+      <c r="C366" s="149" t="n">
         <v>-1.4084E-009</v>
       </c>
       <c r="D366" s="0" t="n">
@@ -22225,7 +22282,7 @@
       <c r="B367" s="0" t="n">
         <v>12</v>
       </c>
-      <c r="C367" s="142" t="n">
+      <c r="C367" s="149" t="n">
         <v>2.0325E-008</v>
       </c>
       <c r="D367" s="0" t="n">
@@ -23986,7 +24043,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:G2383"/>
-  <sheetFormatPr defaultColWidth="11.82421875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.83984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="7.05"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="56.14"/>
@@ -23997,13 +24054,13 @@
       <c r="A1" s="0" t="n">
         <v>3</v>
       </c>
-      <c r="B1" s="143" t="s">
+      <c r="B1" s="150" t="s">
         <v>814</v>
       </c>
-      <c r="C1" s="143" t="n">
+      <c r="C1" s="150" t="n">
         <v>350</v>
       </c>
-      <c r="D1" s="143" t="s">
+      <c r="D1" s="150" t="s">
         <v>815</v>
       </c>
     </row>
@@ -24011,10 +24068,10 @@
       <c r="A2" s="0" t="n">
         <v>2</v>
       </c>
-      <c r="B2" s="143" t="s">
+      <c r="B2" s="150" t="s">
         <v>816</v>
       </c>
-      <c r="C2" s="143" t="n">
+      <c r="C2" s="150" t="n">
         <v>0.5</v>
       </c>
     </row>
@@ -24022,10 +24079,10 @@
       <c r="A3" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="B3" s="143" t="s">
+      <c r="B3" s="150" t="s">
         <v>817</v>
       </c>
-      <c r="C3" s="143" t="n">
+      <c r="C3" s="150" t="n">
         <v>0.0004</v>
       </c>
     </row>
@@ -24129,7 +24186,7 @@
       <c r="B16" s="0" t="s">
         <v>832</v>
       </c>
-      <c r="C16" s="142" t="n">
+      <c r="C16" s="149" t="n">
         <v>3.71179E-009</v>
       </c>
     </row>
@@ -24137,7 +24194,7 @@
       <c r="B17" s="0" t="s">
         <v>833</v>
       </c>
-      <c r="C17" s="142" t="n">
+      <c r="C17" s="149" t="n">
         <v>3.71272E-009</v>
       </c>
     </row>
@@ -24145,7 +24202,7 @@
       <c r="B18" s="0" t="s">
         <v>834</v>
       </c>
-      <c r="C18" s="142" t="n">
+      <c r="C18" s="149" t="n">
         <v>3.71425E-009</v>
       </c>
     </row>
@@ -24153,7 +24210,7 @@
       <c r="B19" s="0" t="s">
         <v>835</v>
       </c>
-      <c r="C19" s="142" t="n">
+      <c r="C19" s="149" t="n">
         <v>3.71562E-009</v>
       </c>
     </row>
@@ -24641,7 +24698,7 @@
       <c r="B80" s="0" t="s">
         <v>903</v>
       </c>
-      <c r="C80" s="142" t="n">
+      <c r="C80" s="149" t="n">
         <v>1.58855E-007</v>
       </c>
     </row>
@@ -24689,7 +24746,7 @@
       <c r="B86" s="0" t="s">
         <v>909</v>
       </c>
-      <c r="C86" s="142" t="n">
+      <c r="C86" s="149" t="n">
         <v>1.58316E-007</v>
       </c>
     </row>
@@ -24721,7 +24778,7 @@
       <c r="B90" s="0" t="s">
         <v>913</v>
       </c>
-      <c r="C90" s="142" t="n">
+      <c r="C90" s="149" t="n">
         <v>1.57838E-007</v>
       </c>
     </row>
@@ -24809,7 +24866,7 @@
       <c r="B101" s="0" t="s">
         <v>925</v>
       </c>
-      <c r="C101" s="142" t="n">
+      <c r="C101" s="149" t="n">
         <v>2.397E-009</v>
       </c>
     </row>
@@ -24985,7 +25042,7 @@
       <c r="B123" s="0" t="s">
         <v>949</v>
       </c>
-      <c r="C123" s="142" t="n">
+      <c r="C123" s="149" t="n">
         <v>2.37898E-010</v>
       </c>
     </row>
@@ -25049,7 +25106,7 @@
       <c r="B131" s="0" t="s">
         <v>957</v>
       </c>
-      <c r="C131" s="142" t="n">
+      <c r="C131" s="149" t="n">
         <v>877987000</v>
       </c>
     </row>
@@ -25065,7 +25122,7 @@
       <c r="B133" s="0" t="s">
         <v>959</v>
       </c>
-      <c r="C133" s="142" t="n">
+      <c r="C133" s="149" t="n">
         <v>1.97895E-005</v>
       </c>
     </row>
@@ -25585,7 +25642,7 @@
       <c r="B198" s="0" t="s">
         <v>1026</v>
       </c>
-      <c r="C198" s="142" t="n">
+      <c r="C198" s="149" t="n">
         <v>2.78422E-007</v>
       </c>
     </row>
@@ -25633,7 +25690,7 @@
       <c r="B204" s="0" t="s">
         <v>1032</v>
       </c>
-      <c r="C204" s="142" t="n">
+      <c r="C204" s="149" t="n">
         <v>2.77565E-007</v>
       </c>
     </row>
@@ -25665,7 +25722,7 @@
       <c r="B208" s="0" t="s">
         <v>1036</v>
       </c>
-      <c r="C208" s="142" t="n">
+      <c r="C208" s="149" t="n">
         <v>2.76716E-007</v>
       </c>
     </row>
@@ -25753,7 +25810,7 @@
       <c r="B219" s="0" t="s">
         <v>1047</v>
       </c>
-      <c r="C219" s="142" t="n">
+      <c r="C219" s="149" t="n">
         <v>5.98328E-009</v>
       </c>
     </row>
@@ -25929,7 +25986,7 @@
       <c r="B241" s="0" t="s">
         <v>1070</v>
       </c>
-      <c r="C241" s="142" t="n">
+      <c r="C241" s="149" t="n">
         <v>4.11728E-010</v>
       </c>
     </row>
@@ -25993,7 +26050,7 @@
       <c r="B249" s="0" t="s">
         <v>1078</v>
       </c>
-      <c r="C249" s="142" t="n">
+      <c r="C249" s="149" t="n">
         <v>877987000</v>
       </c>
     </row>
@@ -26009,7 +26066,7 @@
       <c r="B251" s="0" t="s">
         <v>1080</v>
       </c>
-      <c r="C251" s="142" t="n">
+      <c r="C251" s="149" t="n">
         <v>3.46956E-005</v>
       </c>
     </row>
@@ -26529,7 +26586,7 @@
       <c r="B316" s="0" t="s">
         <v>1145</v>
       </c>
-      <c r="C316" s="142" t="n">
+      <c r="C316" s="149" t="n">
         <v>5.45673E-012</v>
       </c>
     </row>
@@ -26577,7 +26634,7 @@
       <c r="B322" s="0" t="s">
         <v>1151</v>
       </c>
-      <c r="C322" s="142" t="n">
+      <c r="C322" s="149" t="n">
         <v>7.71713E-013</v>
       </c>
     </row>
@@ -26609,7 +26666,7 @@
       <c r="B326" s="0" t="s">
         <v>1155</v>
       </c>
-      <c r="C326" s="142" t="n">
+      <c r="C326" s="149" t="n">
         <v>-7.72781E-012</v>
       </c>
     </row>
@@ -26697,7 +26754,7 @@
       <c r="B337" s="0" t="s">
         <v>1166</v>
       </c>
-      <c r="C337" s="142" t="n">
+      <c r="C337" s="149" t="n">
         <v>5.61762E-010</v>
       </c>
     </row>
@@ -26873,7 +26930,7 @@
       <c r="B359" s="0" t="s">
         <v>1189</v>
       </c>
-      <c r="C359" s="142" t="n">
+      <c r="C359" s="149" t="n">
         <v>2.605E-012</v>
       </c>
     </row>
@@ -26937,7 +26994,7 @@
       <c r="B367" s="0" t="s">
         <v>1197</v>
       </c>
-      <c r="C367" s="142" t="n">
+      <c r="C367" s="149" t="n">
         <v>877987000</v>
       </c>
     </row>
@@ -26953,7 +27010,7 @@
       <c r="B369" s="0" t="s">
         <v>1199</v>
       </c>
-      <c r="C369" s="142" t="n">
+      <c r="C369" s="149" t="n">
         <v>9.64642E-011</v>
       </c>
     </row>
@@ -27473,7 +27530,7 @@
       <c r="B434" s="0" t="s">
         <v>1264</v>
       </c>
-      <c r="C434" s="142" t="n">
+      <c r="C434" s="149" t="n">
         <v>5.42202E-012</v>
       </c>
     </row>
@@ -27521,7 +27578,7 @@
       <c r="B440" s="0" t="s">
         <v>1270</v>
       </c>
-      <c r="C440" s="142" t="n">
+      <c r="C440" s="149" t="n">
         <v>5.83458E-013</v>
       </c>
     </row>
@@ -27553,7 +27610,7 @@
       <c r="B444" s="0" t="s">
         <v>1274</v>
       </c>
-      <c r="C444" s="142" t="n">
+      <c r="C444" s="149" t="n">
         <v>-5.09224E-012</v>
       </c>
     </row>
@@ -27641,7 +27698,7 @@
       <c r="B455" s="0" t="s">
         <v>1285</v>
       </c>
-      <c r="C455" s="142" t="n">
+      <c r="C455" s="149" t="n">
         <v>2.08783E-010</v>
       </c>
     </row>
@@ -27817,7 +27874,7 @@
       <c r="B477" s="0" t="s">
         <v>1308</v>
       </c>
-      <c r="C477" s="142" t="n">
+      <c r="C477" s="149" t="n">
         <v>2.32565E-012</v>
       </c>
     </row>
@@ -27881,7 +27938,7 @@
       <c r="B485" s="0" t="s">
         <v>1316</v>
       </c>
-      <c r="C485" s="142" t="n">
+      <c r="C485" s="149" t="n">
         <v>877987000</v>
       </c>
     </row>
@@ -27897,7 +27954,7 @@
       <c r="B487" s="0" t="s">
         <v>1318</v>
       </c>
-      <c r="C487" s="142" t="n">
+      <c r="C487" s="149" t="n">
         <v>7.29322E-011</v>
       </c>
     </row>
@@ -27985,7 +28042,7 @@
       <c r="B498" s="0" t="s">
         <v>1329</v>
       </c>
-      <c r="C498" s="142" t="n">
+      <c r="C498" s="149" t="n">
         <v>3.71179E-009</v>
       </c>
     </row>
@@ -27993,7 +28050,7 @@
       <c r="B499" s="0" t="s">
         <v>1330</v>
       </c>
-      <c r="C499" s="142" t="n">
+      <c r="C499" s="149" t="n">
         <v>3.71272E-009</v>
       </c>
     </row>
@@ -28001,7 +28058,7 @@
       <c r="B500" s="0" t="s">
         <v>1331</v>
       </c>
-      <c r="C500" s="142" t="n">
+      <c r="C500" s="149" t="n">
         <v>3.71425E-009</v>
       </c>
     </row>
@@ -28009,7 +28066,7 @@
       <c r="B501" s="0" t="s">
         <v>1332</v>
       </c>
-      <c r="C501" s="142" t="n">
+      <c r="C501" s="149" t="n">
         <v>3.71562E-009</v>
       </c>
     </row>
@@ -28577,7 +28634,7 @@
       <c r="B572" s="0" t="s">
         <v>1403</v>
       </c>
-      <c r="C572" s="142" t="n">
+      <c r="C572" s="149" t="n">
         <v>1.19678E-007</v>
       </c>
     </row>
@@ -28625,7 +28682,7 @@
       <c r="B578" s="0" t="s">
         <v>1409</v>
       </c>
-      <c r="C578" s="142" t="n">
+      <c r="C578" s="149" t="n">
         <v>1.19249E-007</v>
       </c>
     </row>
@@ -28657,7 +28714,7 @@
       <c r="B582" s="0" t="s">
         <v>1413</v>
       </c>
-      <c r="C582" s="142" t="n">
+      <c r="C582" s="149" t="n">
         <v>1.18808E-007</v>
       </c>
     </row>
@@ -28745,7 +28802,7 @@
       <c r="B593" s="0" t="s">
         <v>1424</v>
       </c>
-      <c r="C593" s="142" t="n">
+      <c r="C593" s="149" t="n">
         <v>3.58628E-009</v>
       </c>
     </row>
@@ -28921,7 +28978,7 @@
       <c r="B615" s="0" t="s">
         <v>1447</v>
       </c>
-      <c r="C615" s="142" t="n">
+      <c r="C615" s="149" t="n">
         <v>1.9029E-010</v>
       </c>
     </row>
@@ -28985,7 +29042,7 @@
       <c r="B623" s="0" t="s">
         <v>1455</v>
       </c>
-      <c r="C623" s="142" t="n">
+      <c r="C623" s="149" t="n">
         <v>877987000</v>
       </c>
     </row>
@@ -29001,7 +29058,7 @@
       <c r="B625" s="0" t="s">
         <v>1457</v>
       </c>
-      <c r="C625" s="142" t="n">
+      <c r="C625" s="149" t="n">
         <v>1.49062E-005</v>
       </c>
     </row>
@@ -29521,7 +29578,7 @@
       <c r="B690" s="0" t="s">
         <v>1522</v>
       </c>
-      <c r="C690" s="142" t="n">
+      <c r="C690" s="149" t="n">
         <v>5.80654E-012</v>
       </c>
     </row>
@@ -29569,7 +29626,7 @@
       <c r="B696" s="0" t="s">
         <v>1528</v>
       </c>
-      <c r="C696" s="142" t="n">
+      <c r="C696" s="149" t="n">
         <v>-1.88255E-013</v>
       </c>
     </row>
@@ -29601,7 +29658,7 @@
       <c r="B700" s="0" t="s">
         <v>1532</v>
       </c>
-      <c r="C700" s="142" t="n">
+      <c r="C700" s="149" t="n">
         <v>-6.71043E-012</v>
       </c>
     </row>
@@ -29689,7 +29746,7 @@
       <c r="B711" s="0" t="s">
         <v>1543</v>
       </c>
-      <c r="C711" s="142" t="n">
+      <c r="C711" s="149" t="n">
         <v>-3.52979E-010</v>
       </c>
     </row>
@@ -29865,7 +29922,7 @@
       <c r="B733" s="0" t="s">
         <v>1566</v>
       </c>
-      <c r="C733" s="142" t="n">
+      <c r="C733" s="149" t="n">
         <v>2.64443E-012</v>
       </c>
     </row>
@@ -29929,7 +29986,7 @@
       <c r="B741" s="0" t="s">
         <v>1574</v>
       </c>
-      <c r="C741" s="142" t="n">
+      <c r="C741" s="149" t="n">
         <v>877987000</v>
       </c>
     </row>
@@ -29945,7 +30002,7 @@
       <c r="B743" s="0" t="s">
         <v>1576</v>
       </c>
-      <c r="C743" s="142" t="n">
+      <c r="C743" s="149" t="n">
         <v>-2.35319E-011</v>
       </c>
     </row>
@@ -30501,7 +30558,7 @@
       <c r="B811" s="0" t="s">
         <v>1652</v>
       </c>
-      <c r="C811" s="142" t="n">
+      <c r="C811" s="149" t="n">
         <v>877877000</v>
       </c>
     </row>
@@ -31017,7 +31074,7 @@
       <c r="B874" s="0" t="s">
         <v>1717</v>
       </c>
-      <c r="C874" s="142" t="n">
+      <c r="C874" s="149" t="n">
         <v>877877000</v>
       </c>
     </row>
@@ -31533,7 +31590,7 @@
       <c r="B937" s="0" t="s">
         <v>1782</v>
       </c>
-      <c r="C937" s="142" t="n">
+      <c r="C937" s="149" t="n">
         <v>877877000</v>
       </c>
     </row>
@@ -32049,7 +32106,7 @@
       <c r="B1000" s="0" t="s">
         <v>1847</v>
       </c>
-      <c r="C1000" s="142" t="n">
+      <c r="C1000" s="149" t="n">
         <v>877877000</v>
       </c>
     </row>
@@ -32565,7 +32622,7 @@
       <c r="B1063" s="0" t="s">
         <v>1912</v>
       </c>
-      <c r="C1063" s="142" t="n">
+      <c r="C1063" s="149" t="n">
         <v>877877000</v>
       </c>
     </row>
@@ -33081,7 +33138,7 @@
       <c r="B1126" s="0" t="s">
         <v>1977</v>
       </c>
-      <c r="C1126" s="142" t="n">
+      <c r="C1126" s="149" t="n">
         <v>877877000</v>
       </c>
     </row>
@@ -33597,7 +33654,7 @@
       <c r="B1189" s="0" t="s">
         <v>2042</v>
       </c>
-      <c r="C1189" s="142" t="n">
+      <c r="C1189" s="149" t="n">
         <v>877877000</v>
       </c>
     </row>
@@ -34113,7 +34170,7 @@
       <c r="B1252" s="0" t="s">
         <v>2107</v>
       </c>
-      <c r="C1252" s="142" t="n">
+      <c r="C1252" s="149" t="n">
         <v>877877000</v>
       </c>
     </row>
@@ -34629,7 +34686,7 @@
       <c r="B1315" s="0" t="s">
         <v>2172</v>
       </c>
-      <c r="C1315" s="142" t="n">
+      <c r="C1315" s="149" t="n">
         <v>877877000</v>
       </c>
     </row>
@@ -35145,7 +35202,7 @@
       <c r="B1378" s="0" t="s">
         <v>2237</v>
       </c>
-      <c r="C1378" s="142" t="n">
+      <c r="C1378" s="149" t="n">
         <v>877877000</v>
       </c>
     </row>
@@ -35661,7 +35718,7 @@
       <c r="B1441" s="0" t="s">
         <v>2302</v>
       </c>
-      <c r="C1441" s="142" t="n">
+      <c r="C1441" s="149" t="n">
         <v>877877000</v>
       </c>
     </row>
@@ -36109,7 +36166,7 @@
       <c r="B1497" s="0" t="s">
         <v>2361</v>
       </c>
-      <c r="C1497" s="142" t="n">
+      <c r="C1497" s="149" t="n">
         <v>877987000</v>
       </c>
     </row>
@@ -36735,7 +36792,7 @@
       <c r="B1576" s="0" t="s">
         <v>2445</v>
       </c>
-      <c r="C1576" s="142" t="n">
+      <c r="C1576" s="149" t="n">
         <v>877987000</v>
       </c>
     </row>
@@ -36904,7 +36961,7 @@
       <c r="B1596" s="0" t="s">
         <v>2467</v>
       </c>
-      <c r="C1596" s="142" t="n">
+      <c r="C1596" s="149" t="n">
         <v>1000000</v>
       </c>
     </row>
@@ -36912,7 +36969,7 @@
       <c r="B1597" s="0" t="s">
         <v>2468</v>
       </c>
-      <c r="C1597" s="142" t="n">
+      <c r="C1597" s="149" t="n">
         <v>1000000</v>
       </c>
     </row>
@@ -37792,7 +37849,7 @@
       <c r="B1707" s="0" t="s">
         <v>2579</v>
       </c>
-      <c r="C1707" s="142" t="n">
+      <c r="C1707" s="149" t="n">
         <v>877987000</v>
       </c>
     </row>
@@ -37808,7 +37865,7 @@
       <c r="B1709" s="0" t="s">
         <v>2581</v>
       </c>
-      <c r="C1709" s="142" t="n">
+      <c r="C1709" s="149" t="n">
         <v>34197800</v>
       </c>
     </row>
@@ -38328,7 +38385,7 @@
       <c r="B1774" s="0" t="s">
         <v>2646</v>
       </c>
-      <c r="C1774" s="142" t="n">
+      <c r="C1774" s="149" t="n">
         <v>12147700</v>
       </c>
     </row>
@@ -38408,7 +38465,7 @@
       <c r="B1784" s="0" t="s">
         <v>2656</v>
       </c>
-      <c r="C1784" s="142" t="n">
+      <c r="C1784" s="149" t="n">
         <v>-7098040</v>
       </c>
     </row>
@@ -38496,7 +38553,7 @@
       <c r="B1795" s="0" t="s">
         <v>2667</v>
       </c>
-      <c r="C1795" s="142" t="n">
+      <c r="C1795" s="149" t="n">
         <v>4465690</v>
       </c>
     </row>
@@ -38672,7 +38729,7 @@
       <c r="B1817" s="0" t="s">
         <v>2690</v>
       </c>
-      <c r="C1817" s="142" t="n">
+      <c r="C1817" s="149" t="n">
         <v>1999640</v>
       </c>
     </row>
@@ -38736,7 +38793,7 @@
       <c r="B1825" s="0" t="s">
         <v>2698</v>
       </c>
-      <c r="C1825" s="142" t="n">
+      <c r="C1825" s="149" t="n">
         <v>877987000</v>
       </c>
     </row>
@@ -38752,7 +38809,7 @@
       <c r="B1827" s="0" t="s">
         <v>2700</v>
       </c>
-      <c r="C1827" s="142" t="n">
+      <c r="C1827" s="149" t="n">
         <v>-13532400</v>
       </c>
     </row>
@@ -39355,7 +39412,7 @@
       <c r="B1902" s="0" t="s">
         <v>2777</v>
       </c>
-      <c r="C1902" s="142" t="n">
+      <c r="C1902" s="149" t="n">
         <v>4.37265E-007</v>
       </c>
     </row>
@@ -39403,7 +39460,7 @@
       <c r="B1908" s="0" t="s">
         <v>2783</v>
       </c>
-      <c r="C1908" s="142" t="n">
+      <c r="C1908" s="149" t="n">
         <v>4.35882E-007</v>
       </c>
     </row>
@@ -39435,7 +39492,7 @@
       <c r="B1912" s="0" t="s">
         <v>2787</v>
       </c>
-      <c r="C1912" s="142" t="n">
+      <c r="C1912" s="149" t="n">
         <v>4.34577E-007</v>
       </c>
     </row>
@@ -39523,7 +39580,7 @@
       <c r="B1923" s="0" t="s">
         <v>2798</v>
       </c>
-      <c r="C1923" s="142" t="n">
+      <c r="C1923" s="149" t="n">
         <v>9.15083E-009</v>
       </c>
     </row>
@@ -39699,7 +39756,7 @@
       <c r="B1945" s="0" t="s">
         <v>2821</v>
       </c>
-      <c r="C1945" s="142" t="n">
+      <c r="C1945" s="149" t="n">
         <v>6.45121E-010</v>
       </c>
     </row>
@@ -39763,7 +39820,7 @@
       <c r="B1953" s="0" t="s">
         <v>2829</v>
       </c>
-      <c r="C1953" s="142" t="n">
+      <c r="C1953" s="149" t="n">
         <v>877987000</v>
       </c>
     </row>
@@ -39779,7 +39836,7 @@
       <c r="B1955" s="0" t="s">
         <v>2831</v>
       </c>
-      <c r="C1955" s="142" t="n">
+      <c r="C1955" s="149" t="n">
         <v>5.44853E-005</v>
       </c>
     </row>
@@ -40299,7 +40356,7 @@
       <c r="B2020" s="0" t="s">
         <v>2896</v>
       </c>
-      <c r="C2020" s="142" t="n">
+      <c r="C2020" s="149" t="n">
         <v>4.37266E-007</v>
       </c>
     </row>
@@ -40347,7 +40404,7 @@
       <c r="B2026" s="0" t="s">
         <v>2902</v>
       </c>
-      <c r="C2026" s="142" t="n">
+      <c r="C2026" s="149" t="n">
         <v>4.35881E-007</v>
       </c>
     </row>
@@ -40379,7 +40436,7 @@
       <c r="B2030" s="0" t="s">
         <v>2906</v>
       </c>
-      <c r="C2030" s="142" t="n">
+      <c r="C2030" s="149" t="n">
         <v>4.34576E-007</v>
       </c>
     </row>
@@ -40467,7 +40524,7 @@
       <c r="B2041" s="0" t="s">
         <v>2917</v>
       </c>
-      <c r="C2041" s="142" t="n">
+      <c r="C2041" s="149" t="n">
         <v>8.38028E-009</v>
       </c>
     </row>
@@ -40643,7 +40700,7 @@
       <c r="B2063" s="0" t="s">
         <v>2940</v>
       </c>
-      <c r="C2063" s="142" t="n">
+      <c r="C2063" s="149" t="n">
         <v>6.44996E-010</v>
       </c>
     </row>
@@ -40707,7 +40764,7 @@
       <c r="B2071" s="0" t="s">
         <v>2948</v>
       </c>
-      <c r="C2071" s="142" t="n">
+      <c r="C2071" s="149" t="n">
         <v>877987000</v>
       </c>
     </row>
@@ -40723,7 +40780,7 @@
       <c r="B2073" s="0" t="s">
         <v>2950</v>
       </c>
-      <c r="C2073" s="142" t="n">
+      <c r="C2073" s="149" t="n">
         <v>5.44851E-005</v>
       </c>
     </row>
@@ -41243,7 +41300,7 @@
       <c r="B2138" s="0" t="s">
         <v>3015</v>
       </c>
-      <c r="C2138" s="142" t="n">
+      <c r="C2138" s="149" t="n">
         <v>1.0545E-011</v>
       </c>
     </row>
@@ -41291,7 +41348,7 @@
       <c r="B2144" s="0" t="s">
         <v>3021</v>
       </c>
-      <c r="C2144" s="142" t="n">
+      <c r="C2144" s="149" t="n">
         <v>1.35517E-012</v>
       </c>
     </row>
@@ -41323,7 +41380,7 @@
       <c r="B2148" s="0" t="s">
         <v>3025</v>
       </c>
-      <c r="C2148" s="142" t="n">
+      <c r="C2148" s="149" t="n">
         <v>-1.06504E-011</v>
       </c>
     </row>
@@ -41411,7 +41468,7 @@
       <c r="B2159" s="0" t="s">
         <v>3036</v>
       </c>
-      <c r="C2159" s="142" t="n">
+      <c r="C2159" s="149" t="n">
         <v>7.70545E-010</v>
       </c>
     </row>
@@ -41587,7 +41644,7 @@
       <c r="B2181" s="0" t="s">
         <v>3059</v>
       </c>
-      <c r="C2181" s="142" t="n">
+      <c r="C2181" s="149" t="n">
         <v>4.1709E-012</v>
       </c>
     </row>
@@ -41651,7 +41708,7 @@
       <c r="B2189" s="0" t="s">
         <v>3067</v>
       </c>
-      <c r="C2189" s="142" t="n">
+      <c r="C2189" s="149" t="n">
         <v>877987000</v>
       </c>
     </row>
@@ -41667,7 +41724,7 @@
       <c r="B2191" s="0" t="s">
         <v>3069</v>
       </c>
-      <c r="C2191" s="142" t="n">
+      <c r="C2191" s="149" t="n">
         <v>1.69396E-010</v>
       </c>
     </row>
@@ -42243,7 +42300,7 @@
       <c r="B2263" s="0" t="s">
         <v>3144</v>
       </c>
-      <c r="C2263" s="142" t="n">
+      <c r="C2263" s="149" t="n">
         <v>877987000</v>
       </c>
     </row>
@@ -42530,7 +42587,7 @@
       <c r="F2297" s="0" t="s">
         <v>3189</v>
       </c>
-      <c r="G2297" s="144" t="n">
+      <c r="G2297" s="151" t="n">
         <v>41244</v>
       </c>
     </row>
@@ -42622,7 +42679,7 @@
       <c r="B2307" s="0" t="s">
         <v>3203</v>
       </c>
-      <c r="C2307" s="142" t="n">
+      <c r="C2307" s="149" t="n">
         <v>878236000</v>
       </c>
     </row>
@@ -42708,7 +42765,7 @@
       <c r="B2317" s="0" t="s">
         <v>3219</v>
       </c>
-      <c r="C2317" s="142" t="n">
+      <c r="C2317" s="149" t="n">
         <v>32640100000</v>
       </c>
     </row>
@@ -42716,7 +42773,7 @@
       <c r="B2318" s="0" t="s">
         <v>3220</v>
       </c>
-      <c r="C2318" s="142" t="n">
+      <c r="C2318" s="149" t="n">
         <v>33683000000</v>
       </c>
     </row>
@@ -42732,7 +42789,7 @@
       <c r="B2320" s="0" t="s">
         <v>3222</v>
       </c>
-      <c r="C2320" s="142" t="n">
+      <c r="C2320" s="149" t="n">
         <v>30883800</v>
       </c>
     </row>
@@ -42780,7 +42837,7 @@
       <c r="C2326" s="0" t="s">
         <v>3230</v>
       </c>
-      <c r="D2326" s="145" t="n">
+      <c r="D2326" s="152" t="n">
         <v>0.443159722222222</v>
       </c>
     </row>
@@ -42831,7 +42888,7 @@
       <c r="C2332" s="0" t="s">
         <v>3238</v>
       </c>
-      <c r="D2332" s="145" t="n">
+      <c r="D2332" s="152" t="n">
         <v>0.600474537037037</v>
       </c>
     </row>
@@ -42850,7 +42907,7 @@
       <c r="D2334" s="0" t="s">
         <v>3241</v>
       </c>
-      <c r="E2334" s="145" t="n">
+      <c r="E2334" s="152" t="n">
         <v>0.157314814814815</v>
       </c>
     </row>
@@ -42908,7 +42965,7 @@
       <c r="E2339" s="0" t="n">
         <v>30</v>
       </c>
-      <c r="F2339" s="145" t="n">
+      <c r="F2339" s="152" t="n">
         <v>0.596990740740741</v>
       </c>
     </row>
@@ -43380,7 +43437,7 @@
       <c r="E2380" s="0" t="n">
         <v>26</v>
       </c>
-      <c r="F2380" s="145" t="n">
+      <c r="F2380" s="152" t="n">
         <v>0.443159722222222</v>
       </c>
     </row>

</xml_diff>